<commit_message>
ajustando a formula dos estornos
</commit_message>
<xml_diff>
--- a/relatorio_final.xlsx
+++ b/relatorio_final.xlsx
@@ -3154,7 +3154,7 @@
         <v>243.61</v>
       </c>
       <c r="M29" s="81" t="n">
-        <v>0.004557371397943655</v>
+        <v>0.004410035736722273</v>
       </c>
       <c r="N29" s="90" t="n">
         <v>0.05499652205853267</v>
@@ -3183,7 +3183,7 @@
         <v>92147.63333333333</v>
       </c>
       <c r="V29" s="91" t="n">
-        <v>-251.7414155233643</v>
+        <v>-243.6099999999983</v>
       </c>
       <c r="W29" s="75" t="n"/>
     </row>
@@ -3300,7 +3300,7 @@
         <v>443.49</v>
       </c>
       <c r="M31" s="81" t="n">
-        <v>0.004557647473279802</v>
+        <v>0.004410302867216442</v>
       </c>
       <c r="N31" s="90" t="n">
         <v>0.05499993583992224</v>
@@ -3329,7 +3329,7 @@
         <v>97306.78</v>
       </c>
       <c r="V31" s="91" t="n">
-        <v>-455.1479644328822</v>
+        <v>-440.4323654631196</v>
       </c>
       <c r="W31" s="75" t="n"/>
     </row>
@@ -3446,7 +3446,7 @@
         <v>447.48</v>
       </c>
       <c r="M33" s="81" t="n">
-        <v>0.004557687007455069</v>
+        <v>0.004410341120483885</v>
       </c>
       <c r="N33" s="90" t="n">
         <v>0.0550004246965583</v>
@@ -3475,7 +3475,7 @@
         <v>98181.38</v>
       </c>
       <c r="V33" s="91" t="n">
-        <v>-455.1519127992948</v>
+        <v>-440.4361858837273</v>
       </c>
       <c r="W33" s="75" t="n"/>
     </row>
@@ -3519,7 +3519,7 @@
         <v>449.52</v>
       </c>
       <c r="M34" s="81" t="n">
-        <v>0.004557692342789021</v>
+        <v>0.004410346282953004</v>
       </c>
       <c r="N34" s="90" t="n">
         <v>0.05500049067021329</v>
@@ -3548,7 +3548,7 @@
         <v>98628.86</v>
       </c>
       <c r="V34" s="91" t="n">
-        <v>-455.1524456510132</v>
+        <v>-440.4367014685256</v>
       </c>
       <c r="W34" s="75" t="n"/>
     </row>
@@ -3592,7 +3592,7 @@
         <v>407.78</v>
       </c>
       <c r="M35" s="81" t="n">
-        <v>0.004115731403763423</v>
+        <v>0.004410359579613221</v>
       </c>
       <c r="N35" s="90" t="n">
         <v>0.05500066059459408</v>
@@ -3621,7 +3621,7 @@
         <v>99078.38</v>
       </c>
       <c r="V35" s="91" t="n">
-        <v>-371.16139517371</v>
+        <v>-397.7274083609418</v>
       </c>
       <c r="W35" s="75" t="n"/>
     </row>
@@ -3665,7 +3665,7 @@
         <v>453.42</v>
       </c>
       <c r="M36" s="81" t="n">
-        <v>0.004557618868795466</v>
+        <v>0.004410275189517643</v>
       </c>
       <c r="N36" s="90" t="n">
         <v>0.05499958213362155</v>
@@ -3694,7 +3694,7 @@
         <v>99486.16</v>
       </c>
       <c r="V36" s="91" t="n">
-        <v>-455.1451076391307</v>
+        <v>-440.4296012430317</v>
       </c>
       <c r="W36" s="75" t="n"/>
     </row>
@@ -3811,7 +3811,7 @@
         <v>457.5</v>
       </c>
       <c r="M38" s="81" t="n">
-        <v>0.004557665375510833</v>
+        <v>0.004410320189415007</v>
       </c>
       <c r="N38" s="90" t="n">
         <v>0.0550001572084815</v>
@@ -3840,7 +3840,7 @@
         <v>100380.34</v>
       </c>
       <c r="V38" s="91" t="n">
-        <v>-455.1497523686898</v>
+        <v>-440.4340954613273</v>
       </c>
       <c r="W38" s="75" t="n"/>
     </row>
@@ -3957,7 +3957,7 @@
         <v>461.61</v>
       </c>
       <c r="M40" s="81" t="n">
-        <v>0.004557645012364997</v>
+        <v>0.00441030048603519</v>
       </c>
       <c r="N40" s="90" t="n">
         <v>0.0549999054096868</v>
@@ -3986,7 +3986,7 @@
         <v>101282.57</v>
       </c>
       <c r="V40" s="91" t="n">
-        <v>-455.1477186558352</v>
+        <v>-440.4321276504026</v>
       </c>
       <c r="W40" s="75" t="n"/>
     </row>
@@ -4468,7 +4468,7 @@
         <v>464.3</v>
       </c>
       <c r="M47" s="81" t="n">
-        <v>0.004557670066041908</v>
+        <v>0.004410324727972759</v>
       </c>
       <c r="N47" s="90" t="n">
         <v>0.05500021520886333</v>
@@ -4497,7 +4497,7 @@
         <v>101872.2270967742</v>
       </c>
       <c r="V47" s="91" t="n">
-        <v>-455.7533161977407</v>
+        <v>-441.0181451550305</v>
       </c>
       <c r="W47" s="75" t="n"/>
     </row>
@@ -4614,7 +4614,7 @@
         <v>469.54</v>
       </c>
       <c r="M49" s="81" t="n">
-        <v>0.004557680566327216</v>
+        <v>0.00441033488804865</v>
       </c>
       <c r="N49" s="90" t="n">
         <v>0.0550003450493004</v>
@@ -4643,7 +4643,7 @@
         <v>103021.7</v>
       </c>
       <c r="V49" s="91" t="n">
-        <v>-456.8509058466366</v>
+        <v>-442.080248048705</v>
       </c>
       <c r="W49" s="75" t="n"/>
     </row>
@@ -4760,7 +4760,7 @@
         <v>473.76</v>
       </c>
       <c r="M51" s="81" t="n">
-        <v>0.004557677916205316</v>
+        <v>0.004410332323790733</v>
       </c>
       <c r="N51" s="90" t="n">
         <v>0.05500031227942892</v>
@@ -4789,7 +4789,7 @@
         <v>103947.67</v>
       </c>
       <c r="V51" s="91" t="n">
-        <v>-456.8506401846879</v>
+        <v>-442.0799909954671</v>
       </c>
       <c r="W51" s="75" t="n"/>
     </row>
@@ -4833,7 +4833,7 @@
         <v>475.92</v>
       </c>
       <c r="M52" s="81" t="n">
-        <v>0.004557685141833412</v>
+        <v>0.004410339315308542</v>
       </c>
       <c r="N52" s="90" t="n">
         <v>0.05500040162736042</v>
@@ -4862,7 +4862,7 @@
         <v>104421.43</v>
       </c>
       <c r="V52" s="91" t="n">
-        <v>-456.8513645190588</v>
+        <v>-442.0806918579814</v>
       </c>
       <c r="W52" s="75" t="n"/>
     </row>
@@ -4906,7 +4906,7 @@
         <v>431.72</v>
       </c>
       <c r="M53" s="81" t="n">
-        <v>0.004115642578196743</v>
+        <v>0.004410264381438544</v>
       </c>
       <c r="N53" s="90" t="n">
         <v>0.05499944401213863</v>
@@ -4935,7 +4935,7 @@
         <v>104897.35</v>
       </c>
       <c r="V53" s="91" t="n">
-        <v>-372.5393553862689</v>
+        <v>-399.2039954031307</v>
       </c>
       <c r="W53" s="75" t="n"/>
     </row>
@@ -4979,7 +4979,7 @@
         <v>480.05</v>
       </c>
       <c r="M54" s="81" t="n">
-        <v>0.004557621177135651</v>
+        <v>0.004410277423067432</v>
       </c>
       <c r="N54" s="90" t="n">
         <v>0.05499961067720038</v>
@@ -5008,7 +5008,7 @@
         <v>105329.07</v>
       </c>
       <c r="V54" s="91" t="n">
-        <v>-456.8449523664911</v>
+        <v>-442.0744874895442</v>
       </c>
       <c r="W54" s="75" t="n"/>
     </row>
@@ -5563,7 +5563,7 @@
         <v>477.18</v>
       </c>
       <c r="M62" s="81" t="n">
-        <v>0.004557786755774007</v>
+        <v>0.004410437636956255</v>
       </c>
       <c r="N62" s="90" t="n">
         <v>0.05500165812722302</v>
@@ -5592,7 +5592,7 @@
         <v>104695.5519354839</v>
       </c>
       <c r="V62" s="91" t="n">
-        <v>-449.4186127781232</v>
+        <v>-434.8882511153035</v>
       </c>
       <c r="W62" s="75" t="n"/>
     </row>
@@ -5709,7 +5709,7 @@
         <v>433.37</v>
       </c>
       <c r="M64" s="81" t="n">
-        <v>0.004557672695852277</v>
+        <v>0.004410327272577286</v>
       </c>
       <c r="N64" s="90" t="n">
         <v>0.05500024772757151</v>
@@ -5738,7 +5738,7 @@
         <v>95085.81</v>
       </c>
       <c r="V64" s="91" t="n">
-        <v>-399.9319442075342</v>
+        <v>-387.0015597174782</v>
       </c>
       <c r="W64" s="75" t="n"/>
     </row>
@@ -6220,7 +6220,7 @@
         <v>435.92</v>
       </c>
       <c r="M71" s="81" t="n">
-        <v>0.004557592194033067</v>
+        <v>0.004410249379017683</v>
       </c>
       <c r="N71" s="90" t="n">
         <v>0.05499925228922997</v>
@@ -6249,7 +6249,7 @@
         <v>95646.99548387097</v>
       </c>
       <c r="V71" s="91" t="n">
-        <v>-400.5268739092156</v>
+        <v>-387.577254990522</v>
       </c>
       <c r="W71" s="75" t="n"/>
     </row>
@@ -6366,7 +6366,7 @@
         <v>440.77</v>
       </c>
       <c r="M73" s="81" t="n">
-        <v>0.004557649399844488</v>
+        <v>0.004410304731360393</v>
       </c>
       <c r="N73" s="90" t="n">
         <v>0.05499995966269666</v>
@@ -6395,7 +6395,7 @@
         <v>96709.94</v>
       </c>
       <c r="V73" s="91" t="n">
-        <v>-401.4850710615175</v>
+        <v>-388.5044718598697</v>
       </c>
       <c r="W73" s="75" t="n"/>
     </row>
@@ -6512,7 +6512,7 @@
         <v>444.73</v>
       </c>
       <c r="M75" s="81" t="n">
-        <v>0.004557632535714395</v>
+        <v>0.004410288413628116</v>
       </c>
       <c r="N75" s="90" t="n">
         <v>0.05515451658257575</v>
@@ -6541,7 +6541,7 @@
         <v>97579.17</v>
       </c>
       <c r="V75" s="91" t="n">
-        <v>-401.4835853813657</v>
+        <v>-388.5030343228018</v>
       </c>
       <c r="W75" s="75" t="n"/>
     </row>
@@ -6585,7 +6585,7 @@
         <v>445.54</v>
       </c>
       <c r="M76" s="81" t="n">
-        <v>0.004545218053964462</v>
+        <v>0.004398276158800174</v>
       </c>
       <c r="N76" s="90" t="n">
         <v>0.05500057349558163</v>
@@ -6614,7 +6614,7 @@
         <v>98023.89999999999</v>
       </c>
       <c r="V76" s="91" t="n">
-        <v>-400.3899063617669</v>
+        <v>-387.4447954692743</v>
       </c>
       <c r="W76" s="75" t="n"/>
     </row>
@@ -6658,7 +6658,7 @@
         <v>418.62</v>
       </c>
       <c r="M77" s="81" t="n">
-        <v>0.004251268210726078</v>
+        <v>0.004398185579549407</v>
       </c>
       <c r="N77" s="90" t="n">
         <v>0.05499941275525555</v>
@@ -6687,7 +6687,7 @@
         <v>98469.44</v>
       </c>
       <c r="V77" s="91" t="n">
-        <v>-350.2834584595251</v>
+        <v>-362.3878376864934</v>
       </c>
       <c r="W77" s="75" t="n"/>
     </row>
@@ -6731,7 +6731,7 @@
         <v>449.46</v>
       </c>
       <c r="M78" s="81" t="n">
-        <v>0.004545139221054484</v>
+        <v>0.00439819988004686</v>
       </c>
       <c r="N78" s="90" t="n">
         <v>0.05499959601087667</v>
@@ -6760,7 +6760,7 @@
         <v>98888.06</v>
       </c>
       <c r="V78" s="91" t="n">
-        <v>-400.3829614176663</v>
+        <v>-387.4380755715193</v>
       </c>
       <c r="W78" s="75" t="n"/>
     </row>
@@ -6877,7 +6877,7 @@
         <v>233.8</v>
       </c>
       <c r="M80" s="81" t="n">
-        <v>0.004545102829229819</v>
+        <v>0.004398164667303472</v>
       </c>
       <c r="N80" s="90" t="n">
         <v>0.05499914477255552</v>
@@ -6888,13 +6888,13 @@
         </is>
       </c>
       <c r="P80" s="88" t="n">
-        <v>-13909.23327915017</v>
+        <v>-13705.39765423249</v>
       </c>
       <c r="Q80" s="83" t="n">
         <v>233.8</v>
       </c>
       <c r="R80" s="91" t="n">
-        <v>-71333.05672084983</v>
+        <v>-71536.8923457675</v>
       </c>
       <c r="S80" s="84" t="n">
         <v>-0</v>
@@ -6906,7 +6906,7 @@
         <v>99774.42999999999</v>
       </c>
       <c r="V80" s="91" t="n">
-        <v>-206.4133332362132</v>
+        <v>-199.7470434258513</v>
       </c>
       <c r="W80" s="75" t="n"/>
     </row>
@@ -6967,7 +6967,7 @@
         <v>0</v>
       </c>
       <c r="R81" s="91" t="n">
-        <v>28675.17327915017</v>
+        <v>28471.3376542325</v>
       </c>
       <c r="S81" s="84" t="n">
         <v>0</v>
@@ -7040,7 +7040,7 @@
         <v>0</v>
       </c>
       <c r="R82" s="91" t="n">
-        <v>-71333.05672084983</v>
+        <v>-71536.8923457675</v>
       </c>
       <c r="S82" s="84" t="n">
         <v>-1500123.45</v>
@@ -7096,7 +7096,7 @@
         <v>219.69</v>
       </c>
       <c r="M83" s="81" t="n">
-        <v>0.004545205483181158</v>
+        <v>0.004398263995305518</v>
       </c>
       <c r="N83" s="90" t="n">
         <v>0.05500041762472985</v>
@@ -7113,7 +7113,7 @@
         <v>219.69</v>
       </c>
       <c r="R83" s="91" t="n">
-        <v>-71333.05672084983</v>
+        <v>-71536.8923457675</v>
       </c>
       <c r="S83" s="84" t="n">
         <v>-3006837.6</v>
@@ -7186,7 +7186,7 @@
         <v>440.83</v>
       </c>
       <c r="R84" s="91" t="n">
-        <v>-71333.05672084983</v>
+        <v>-71536.8923457675</v>
       </c>
       <c r="S84" s="84" t="n">
         <v>-3120731.25</v>
@@ -7242,7 +7242,7 @@
         <v>457.56</v>
       </c>
       <c r="M85" s="81" t="n">
-        <v>0.004545203948593812</v>
+        <v>0.0043982625104384</v>
       </c>
       <c r="N85" s="90" t="n">
         <v>0.05500039859668648</v>
@@ -7259,7 +7259,7 @@
         <v>457.56</v>
       </c>
       <c r="R85" s="91" t="n">
-        <v>-71333.05672084983</v>
+        <v>-71536.8923457675</v>
       </c>
       <c r="S85" s="84" t="n">
         <v>-1719147.27</v>
@@ -7332,7 +7332,7 @@
         <v>0</v>
       </c>
       <c r="R86" s="91" t="n">
-        <v>-71588.95672084982</v>
+        <v>-71792.79234576749</v>
       </c>
       <c r="S86" s="84" t="n">
         <v>-0</v>
@@ -7405,7 +7405,7 @@
         <v>0</v>
       </c>
       <c r="R87" s="91" t="n">
-        <v>-71663.24672084981</v>
+        <v>-71867.08234576749</v>
       </c>
       <c r="S87" s="84" t="n">
         <v>-1420391</v>
@@ -7461,7 +7461,7 @@
         <v>460.31</v>
       </c>
       <c r="M88" s="81" t="n">
-        <v>0.004545130134693265</v>
+        <v>0.00439819108808015</v>
       </c>
       <c r="N88" s="90" t="n">
         <v>0.05499948334505067</v>
@@ -7478,7 +7478,7 @@
         <v>460.31</v>
       </c>
       <c r="R88" s="91" t="n">
-        <v>-71663.24672084981</v>
+        <v>-71867.08234576749</v>
       </c>
       <c r="S88" s="84" t="n">
         <v>-3057504.3</v>
@@ -7551,7 +7551,7 @@
         <v>448.25</v>
       </c>
       <c r="R89" s="91" t="n">
-        <v>-71663.24672084981</v>
+        <v>-71867.08234576749</v>
       </c>
       <c r="S89" s="84" t="n">
         <v>-3173316.86</v>
@@ -7607,7 +7607,7 @@
         <v>465.27</v>
       </c>
       <c r="M90" s="81" t="n">
-        <v>0.004545203216800742</v>
+        <v>0.00439826180235503</v>
       </c>
       <c r="N90" s="90" t="n">
         <v>0.05500038952285258</v>
@@ -7624,7 +7624,7 @@
         <v>465.27</v>
       </c>
       <c r="R90" s="91" t="n">
-        <v>-71663.24672084981</v>
+        <v>-71867.08234576749</v>
       </c>
       <c r="S90" s="84" t="n">
         <v>-3084909.9</v>
@@ -7697,7 +7697,7 @@
         <v>452.27</v>
       </c>
       <c r="R91" s="91" t="n">
-        <v>-71663.24672084981</v>
+        <v>-71867.08234576749</v>
       </c>
       <c r="S91" s="84" t="n">
         <v>-3201760.6</v>
@@ -7753,7 +7753,7 @@
         <v>469.44</v>
       </c>
       <c r="M92" s="81" t="n">
-        <v>0.004545199288166657</v>
+        <v>0.004398258001007127</v>
       </c>
       <c r="N92" s="90" t="n">
         <v>0.05484601912472131</v>
@@ -7770,7 +7770,7 @@
         <v>469.44</v>
       </c>
       <c r="R92" s="91" t="n">
-        <v>-71663.24672084981</v>
+        <v>-71867.08234576749</v>
       </c>
       <c r="S92" s="84" t="n">
         <v>-3216313.24</v>
@@ -7826,7 +7826,7 @@
         <v>472.87</v>
       </c>
       <c r="M93" s="81" t="n">
-        <v>0.00455769351619506</v>
+        <v>0.004410347418340788</v>
       </c>
       <c r="N93" s="90" t="n">
         <v>0.05500050517987431</v>
@@ -7843,7 +7843,7 @@
         <v>472.87</v>
       </c>
       <c r="R93" s="91" t="n">
-        <v>-71663.24672084981</v>
+        <v>-71867.08234576749</v>
       </c>
       <c r="S93" s="84" t="n">
         <v>-312674.73</v>
@@ -7902,7 +7902,7 @@
         <v>0.0008333382603676356</v>
       </c>
       <c r="N94" s="90" t="n">
-        <v>0.01019037987659588</v>
+        <v>0.009373418609034623</v>
       </c>
       <c r="O94" s="82" t="inlineStr">
         <is>
@@ -7916,7 +7916,7 @@
         <v>0</v>
       </c>
       <c r="R94" s="91" t="n">
-        <v>-72393.86672084981</v>
+        <v>-72597.70234576748</v>
       </c>
       <c r="S94" s="84" t="n">
         <v>-0</v>
@@ -7972,7 +7972,7 @@
         <v>45.88</v>
       </c>
       <c r="M95" s="81" t="n">
-        <v>0.004116094674724957</v>
+        <v>0.004410748912710316</v>
       </c>
       <c r="N95" s="90" t="n">
         <v>0.0550056360796074</v>
@@ -7989,7 +7989,7 @@
         <v>45.88</v>
       </c>
       <c r="R95" s="91" t="n">
-        <v>-72393.86672084981</v>
+        <v>-72597.70234576748</v>
       </c>
       <c r="S95" s="84" t="n">
         <v>-0</v>
@@ -8062,7 +8062,7 @@
         <v>0</v>
       </c>
       <c r="R96" s="91" t="n">
-        <v>-74493.89672084981</v>
+        <v>-74697.73234576748</v>
       </c>
       <c r="S96" s="84" t="n">
         <v>-0</v>

</xml_diff>

<commit_message>
Correção na templete 'laudo_completo' para recebimento de informações
</commit_message>
<xml_diff>
--- a/relatorio_final.xlsx
+++ b/relatorio_final.xlsx
@@ -2511,10 +2511,10 @@
         <v>0</v>
       </c>
       <c r="Q20" s="83" t="n">
-        <v>0</v>
+        <v>305.66</v>
       </c>
       <c r="R20" s="91" t="n">
-        <v>-56547.16</v>
+        <v>-56241.5</v>
       </c>
       <c r="S20" s="84" t="n">
         <v>-0</v>
@@ -2584,10 +2584,10 @@
         <v>0</v>
       </c>
       <c r="Q21" s="83" t="n">
-        <v>0</v>
+        <v>88.73999999999999</v>
       </c>
       <c r="R21" s="91" t="n">
-        <v>-56635.9</v>
+        <v>-56241.5</v>
       </c>
       <c r="S21" s="84" t="n">
         <v>-0</v>
@@ -2660,7 +2660,7 @@
         <v>0</v>
       </c>
       <c r="R22" s="91" t="n">
-        <v>-56637.06</v>
+        <v>-56242.66</v>
       </c>
       <c r="S22" s="84" t="n">
         <v>-0</v>
@@ -2733,7 +2733,7 @@
         <v>0</v>
       </c>
       <c r="R23" s="91" t="n">
-        <v>-56637.4</v>
+        <v>-56243</v>
       </c>
       <c r="S23" s="84" t="n">
         <v>-0</v>
@@ -2806,7 +2806,7 @@
         <v>0</v>
       </c>
       <c r="R24" s="91" t="n">
-        <v>-56636.24</v>
+        <v>-56241.84</v>
       </c>
       <c r="S24" s="84" t="n">
         <v>-0</v>
@@ -2879,7 +2879,7 @@
         <v>0</v>
       </c>
       <c r="R25" s="91" t="n">
-        <v>-56635.9</v>
+        <v>-56241.5</v>
       </c>
       <c r="S25" s="84" t="n">
         <v>-0</v>
@@ -2952,7 +2952,7 @@
         <v>0</v>
       </c>
       <c r="R26" s="91" t="n">
-        <v>-96635.89999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S26" s="84" t="n">
         <v>-0</v>
@@ -3025,7 +3025,7 @@
         <v>0</v>
       </c>
       <c r="R27" s="91" t="n">
-        <v>-96787.89999999999</v>
+        <v>-96393.5</v>
       </c>
       <c r="S27" s="84" t="n">
         <v>-0</v>
@@ -3098,7 +3098,7 @@
         <v>0</v>
       </c>
       <c r="R28" s="91" t="n">
-        <v>-96635.89999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S28" s="84" t="n">
         <v>-1546174.4</v>
@@ -3154,7 +3154,7 @@
         <v>243.61</v>
       </c>
       <c r="M29" s="81" t="n">
-        <v>0.004410035736722273</v>
+        <v>0.004557371397943655</v>
       </c>
       <c r="N29" s="90" t="n">
         <v>0.05499652205853267</v>
@@ -3171,7 +3171,7 @@
         <v>243.61</v>
       </c>
       <c r="R29" s="91" t="n">
-        <v>-96635.89999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S29" s="84" t="n">
         <v>-2906385.3</v>
@@ -3183,7 +3183,7 @@
         <v>92147.63333333333</v>
       </c>
       <c r="V29" s="91" t="n">
-        <v>-243.6099999999983</v>
+        <v>-250.7836595524696</v>
       </c>
       <c r="W29" s="75" t="n"/>
     </row>
@@ -3244,7 +3244,7 @@
         <v>427.27</v>
       </c>
       <c r="R30" s="91" t="n">
-        <v>-96635.89999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S30" s="84" t="n">
         <v>-3016510.18</v>
@@ -3256,7 +3256,7 @@
         <v>96879.50999999999</v>
       </c>
       <c r="V30" s="91" t="n">
-        <v>-426.1956010409145</v>
+        <v>-424.4561693695529</v>
       </c>
       <c r="W30" s="75" t="n"/>
     </row>
@@ -3300,7 +3300,7 @@
         <v>443.49</v>
       </c>
       <c r="M31" s="81" t="n">
-        <v>0.004410302867216442</v>
+        <v>0.004557647473279802</v>
       </c>
       <c r="N31" s="90" t="n">
         <v>0.05499993583992224</v>
@@ -3317,7 +3317,7 @@
         <v>443.49</v>
       </c>
       <c r="R31" s="91" t="n">
-        <v>-96635.89999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S31" s="84" t="n">
         <v>-2932508.1</v>
@@ -3329,7 +3329,7 @@
         <v>97306.78</v>
       </c>
       <c r="V31" s="91" t="n">
-        <v>-440.4323654631196</v>
+        <v>-453.2903695103708</v>
       </c>
       <c r="W31" s="75" t="n"/>
     </row>
@@ -3390,7 +3390,7 @@
         <v>431.11</v>
       </c>
       <c r="R32" s="91" t="n">
-        <v>-96635.89999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S32" s="84" t="n">
         <v>-3043622.78</v>
@@ -3402,7 +3402,7 @@
         <v>97750.27</v>
       </c>
       <c r="V32" s="91" t="n">
-        <v>-426.1952713685529</v>
+        <v>-424.4558410426828</v>
       </c>
       <c r="W32" s="75" t="n"/>
     </row>
@@ -3446,7 +3446,7 @@
         <v>447.48</v>
       </c>
       <c r="M33" s="81" t="n">
-        <v>0.004410341120483885</v>
+        <v>0.004557687007455069</v>
       </c>
       <c r="N33" s="90" t="n">
         <v>0.0550004246965583</v>
@@ -3463,7 +3463,7 @@
         <v>447.48</v>
       </c>
       <c r="R33" s="91" t="n">
-        <v>-96635.89999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S33" s="84" t="n">
         <v>-3057494.66</v>
@@ -3475,7 +3475,7 @@
         <v>98181.38</v>
       </c>
       <c r="V33" s="91" t="n">
-        <v>-440.4361858837273</v>
+        <v>-453.2943017623195</v>
       </c>
       <c r="W33" s="75" t="n"/>
     </row>
@@ -3519,7 +3519,7 @@
         <v>449.52</v>
       </c>
       <c r="M34" s="81" t="n">
-        <v>0.004410346282953004</v>
+        <v>0.004557692342789021</v>
       </c>
       <c r="N34" s="90" t="n">
         <v>0.05500049067021329</v>
@@ -3536,7 +3536,7 @@
         <v>449.52</v>
       </c>
       <c r="R34" s="91" t="n">
-        <v>-96635.89999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S34" s="84" t="n">
         <v>-2774194.64</v>
@@ -3548,7 +3548,7 @@
         <v>98628.86</v>
       </c>
       <c r="V34" s="91" t="n">
-        <v>-440.4367014685256</v>
+        <v>-453.2948324393108</v>
       </c>
       <c r="W34" s="75" t="n"/>
     </row>
@@ -3592,7 +3592,7 @@
         <v>407.78</v>
       </c>
       <c r="M35" s="81" t="n">
-        <v>0.004410359579613221</v>
+        <v>0.004115731403763423</v>
       </c>
       <c r="N35" s="90" t="n">
         <v>0.05500066059459408</v>
@@ -3609,7 +3609,7 @@
         <v>407.78</v>
       </c>
       <c r="R35" s="91" t="n">
-        <v>-96635.89999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S35" s="84" t="n">
         <v>-3084070.96</v>
@@ -3621,7 +3621,7 @@
         <v>99078.38</v>
       </c>
       <c r="V35" s="91" t="n">
-        <v>-397.7274083609418</v>
+        <v>-369.6465745505615</v>
       </c>
       <c r="W35" s="75" t="n"/>
     </row>
@@ -3665,7 +3665,7 @@
         <v>453.42</v>
       </c>
       <c r="M36" s="81" t="n">
-        <v>0.004410275189517643</v>
+        <v>0.004557618868795466</v>
       </c>
       <c r="N36" s="90" t="n">
         <v>0.05499958213362155</v>
@@ -3682,7 +3682,7 @@
         <v>453.42</v>
       </c>
       <c r="R36" s="91" t="n">
-        <v>-96635.89999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S36" s="84" t="n">
         <v>-2998187.4</v>
@@ -3694,7 +3694,7 @@
         <v>99486.16</v>
       </c>
       <c r="V36" s="91" t="n">
-        <v>-440.4296012430317</v>
+        <v>-453.2875243760486</v>
       </c>
       <c r="W36" s="75" t="n"/>
     </row>
@@ -3755,7 +3755,7 @@
         <v>440.76</v>
       </c>
       <c r="R37" s="91" t="n">
-        <v>-96635.89999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S37" s="84" t="n">
         <v>-3111790.54</v>
@@ -3767,7 +3767,7 @@
         <v>99939.58</v>
       </c>
       <c r="V37" s="91" t="n">
-        <v>-426.1898967756351</v>
+        <v>-424.4504883850855</v>
       </c>
       <c r="W37" s="75" t="n"/>
     </row>
@@ -3811,7 +3811,7 @@
         <v>457.5</v>
       </c>
       <c r="M38" s="81" t="n">
-        <v>0.004410320189415007</v>
+        <v>0.004557665375510833</v>
       </c>
       <c r="N38" s="90" t="n">
         <v>0.0550001572084815</v>
@@ -3828,7 +3828,7 @@
         <v>457.5</v>
       </c>
       <c r="R38" s="91" t="n">
-        <v>-96635.89999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S38" s="84" t="n">
         <v>-3025135.2</v>
@@ -3840,7 +3840,7 @@
         <v>100380.34</v>
       </c>
       <c r="V38" s="91" t="n">
-        <v>-440.4340954613273</v>
+        <v>-453.2921501490778</v>
       </c>
       <c r="W38" s="75" t="n"/>
     </row>
@@ -3901,7 +3901,7 @@
         <v>444.73</v>
       </c>
       <c r="R39" s="91" t="n">
-        <v>-96635.89999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S39" s="84" t="n">
         <v>-3139759.67</v>
@@ -3913,7 +3913,7 @@
         <v>100837.84</v>
       </c>
       <c r="V39" s="91" t="n">
-        <v>-426.197980906763</v>
+        <v>-424.4585395224573</v>
       </c>
       <c r="W39" s="75" t="n"/>
     </row>
@@ -3957,7 +3957,7 @@
         <v>461.61</v>
       </c>
       <c r="M40" s="81" t="n">
-        <v>0.00441030048603519</v>
+        <v>0.004557645012364997</v>
       </c>
       <c r="N40" s="90" t="n">
         <v>0.0549999054096868</v>
@@ -3974,7 +3974,7 @@
         <v>461.61</v>
       </c>
       <c r="R40" s="91" t="n">
-        <v>-96635.89999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S40" s="84" t="n">
         <v>-2034883.6</v>
@@ -3986,7 +3986,7 @@
         <v>101282.57</v>
       </c>
       <c r="V40" s="91" t="n">
-        <v>-440.4321276504026</v>
+        <v>-453.2901247364134</v>
       </c>
       <c r="W40" s="75" t="n"/>
     </row>
@@ -4044,10 +4044,10 @@
         <v>0</v>
       </c>
       <c r="Q41" s="83" t="n">
-        <v>0</v>
+        <v>279.67</v>
       </c>
       <c r="R41" s="91" t="n">
-        <v>-96915.56999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S41" s="84" t="n">
         <v>-0</v>
@@ -4117,10 +4117,10 @@
         <v>0</v>
       </c>
       <c r="Q42" s="83" t="n">
-        <v>0</v>
+        <v>81.19</v>
       </c>
       <c r="R42" s="91" t="n">
-        <v>-96996.75999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S42" s="84" t="n">
         <v>-0</v>
@@ -4193,7 +4193,7 @@
         <v>0</v>
       </c>
       <c r="R43" s="91" t="n">
-        <v>-96997.81999999999</v>
+        <v>-96242.56</v>
       </c>
       <c r="S43" s="84" t="n">
         <v>-0</v>
@@ -4266,7 +4266,7 @@
         <v>0</v>
       </c>
       <c r="R44" s="91" t="n">
-        <v>-96998.12999999999</v>
+        <v>-96242.87</v>
       </c>
       <c r="S44" s="84" t="n">
         <v>-0</v>
@@ -4339,7 +4339,7 @@
         <v>0</v>
       </c>
       <c r="R45" s="91" t="n">
-        <v>-96997.06999999999</v>
+        <v>-96241.81</v>
       </c>
       <c r="S45" s="84" t="n">
         <v>-0</v>
@@ -4412,7 +4412,7 @@
         <v>0</v>
       </c>
       <c r="R46" s="91" t="n">
-        <v>-96996.75999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S46" s="84" t="n">
         <v>-1123155.44</v>
@@ -4468,7 +4468,7 @@
         <v>464.3</v>
       </c>
       <c r="M47" s="81" t="n">
-        <v>0.004410324727972759</v>
+        <v>0.004557670066041908</v>
       </c>
       <c r="N47" s="90" t="n">
         <v>0.05500021520886333</v>
@@ -4485,7 +4485,7 @@
         <v>464.3</v>
       </c>
       <c r="R47" s="91" t="n">
-        <v>-96996.75999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S47" s="84" t="n">
         <v>-3077080.2</v>
@@ -4497,7 +4497,7 @@
         <v>101872.2270967742</v>
       </c>
       <c r="V47" s="91" t="n">
-        <v>-441.0181451550305</v>
+        <v>-453.2926166909854</v>
       </c>
       <c r="W47" s="75" t="n"/>
     </row>
@@ -4558,7 +4558,7 @@
         <v>452.36</v>
       </c>
       <c r="R48" s="91" t="n">
-        <v>-96996.75999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S48" s="84" t="n">
         <v>-3193672.7</v>
@@ -4570,7 +4570,7 @@
         <v>102569.34</v>
       </c>
       <c r="V48" s="91" t="n">
-        <v>-427.7833351915854</v>
+        <v>-424.4524235019908</v>
       </c>
       <c r="W48" s="75" t="n"/>
     </row>
@@ -4614,7 +4614,7 @@
         <v>469.54</v>
       </c>
       <c r="M49" s="81" t="n">
-        <v>0.00441033488804865</v>
+        <v>0.004557680566327216</v>
       </c>
       <c r="N49" s="90" t="n">
         <v>0.0550003450493004</v>
@@ -4631,7 +4631,7 @@
         <v>469.54</v>
       </c>
       <c r="R49" s="91" t="n">
-        <v>-96996.75999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S49" s="84" t="n">
         <v>-3104737.2</v>
@@ -4643,7 +4643,7 @@
         <v>103021.7</v>
       </c>
       <c r="V49" s="91" t="n">
-        <v>-442.080248048705</v>
+        <v>-453.2936610979489</v>
       </c>
       <c r="W49" s="75" t="n"/>
     </row>
@@ -4704,7 +4704,7 @@
         <v>456.43</v>
       </c>
       <c r="R50" s="91" t="n">
-        <v>-96996.75999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S50" s="84" t="n">
         <v>-3222377.77</v>
@@ -4716,7 +4716,7 @@
         <v>103491.24</v>
       </c>
       <c r="V50" s="91" t="n">
-        <v>-427.7872326855828</v>
+        <v>-424.4562906483631</v>
       </c>
       <c r="W50" s="75" t="n"/>
     </row>
@@ -4760,7 +4760,7 @@
         <v>473.76</v>
       </c>
       <c r="M51" s="81" t="n">
-        <v>0.004410332323790733</v>
+        <v>0.004557677916205316</v>
       </c>
       <c r="N51" s="90" t="n">
         <v>0.05500031227942892</v>
@@ -4777,7 +4777,7 @@
         <v>473.76</v>
       </c>
       <c r="R51" s="91" t="n">
-        <v>-96996.75999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S51" s="84" t="n">
         <v>-3237064.33</v>
@@ -4789,7 +4789,7 @@
         <v>103947.67</v>
       </c>
       <c r="V51" s="91" t="n">
-        <v>-442.0799909954671</v>
+        <v>-453.2933975045624</v>
       </c>
       <c r="W51" s="75" t="n"/>
     </row>
@@ -4833,7 +4833,7 @@
         <v>475.92</v>
       </c>
       <c r="M52" s="81" t="n">
-        <v>0.004410339315308542</v>
+        <v>0.004557685141833412</v>
       </c>
       <c r="N52" s="90" t="n">
         <v>0.05500040162736042</v>
@@ -4850,7 +4850,7 @@
         <v>475.92</v>
       </c>
       <c r="R52" s="91" t="n">
-        <v>-96996.75999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S52" s="84" t="n">
         <v>-2937125.8</v>
@@ -4862,7 +4862,7 @@
         <v>104421.43</v>
       </c>
       <c r="V52" s="91" t="n">
-        <v>-442.0806918579814</v>
+        <v>-453.2941161989432</v>
       </c>
       <c r="W52" s="75" t="n"/>
     </row>
@@ -4906,7 +4906,7 @@
         <v>431.72</v>
       </c>
       <c r="M53" s="81" t="n">
-        <v>0.004410264381438544</v>
+        <v>0.004115642578196743</v>
       </c>
       <c r="N53" s="90" t="n">
         <v>0.05499944401213863</v>
@@ -4923,7 +4923,7 @@
         <v>431.72</v>
       </c>
       <c r="R53" s="91" t="n">
-        <v>-96996.75999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S53" s="84" t="n">
         <v>-3265201.17</v>
@@ -4935,7 +4935,7 @@
         <v>104897.35</v>
       </c>
       <c r="V53" s="91" t="n">
-        <v>-399.2039954031307</v>
+        <v>-369.6385979429375</v>
       </c>
       <c r="W53" s="75" t="n"/>
     </row>
@@ -4979,7 +4979,7 @@
         <v>480.05</v>
       </c>
       <c r="M54" s="81" t="n">
-        <v>0.004410277423067432</v>
+        <v>0.004557621177135651</v>
       </c>
       <c r="N54" s="90" t="n">
         <v>0.05499961067720038</v>
@@ -4996,7 +4996,7 @@
         <v>480.05</v>
       </c>
       <c r="R54" s="91" t="n">
-        <v>-96996.75999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S54" s="84" t="n">
         <v>-3174273.6</v>
@@ -5008,7 +5008,7 @@
         <v>105329.07</v>
       </c>
       <c r="V54" s="91" t="n">
-        <v>-442.0744874895442</v>
+        <v>-453.2877539742529</v>
       </c>
       <c r="W54" s="75" t="n"/>
     </row>
@@ -5069,7 +5069,7 @@
         <v>466.65</v>
       </c>
       <c r="R55" s="91" t="n">
-        <v>-96996.75999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S55" s="84" t="n">
         <v>-1700412.32</v>
@@ -5081,7 +5081,7 @@
         <v>105809.12</v>
       </c>
       <c r="V55" s="91" t="n">
-        <v>-427.7848455218292</v>
+        <v>-424.4539220721303</v>
       </c>
       <c r="W55" s="75" t="n"/>
     </row>
@@ -5142,7 +5142,7 @@
         <v>0</v>
       </c>
       <c r="R56" s="91" t="n">
-        <v>-96937.84</v>
+        <v>-96182.58</v>
       </c>
       <c r="S56" s="84" t="n">
         <v>-1168385.35</v>
@@ -5215,7 +5215,7 @@
         <v>0</v>
       </c>
       <c r="R57" s="91" t="n">
-        <v>-96853.92999999999</v>
+        <v>-96098.67</v>
       </c>
       <c r="S57" s="84" t="n">
         <v>-0</v>
@@ -5288,7 +5288,7 @@
         <v>0</v>
       </c>
       <c r="R58" s="91" t="n">
-        <v>-90604.87</v>
+        <v>-89849.61</v>
       </c>
       <c r="S58" s="84" t="n">
         <v>-0</v>
@@ -5361,7 +5361,7 @@
         <v>0</v>
       </c>
       <c r="R59" s="91" t="n">
-        <v>-89896.33</v>
+        <v>-89141.07000000001</v>
       </c>
       <c r="S59" s="84" t="n">
         <v>-0</v>
@@ -5434,7 +5434,7 @@
         <v>0</v>
       </c>
       <c r="R60" s="91" t="n">
-        <v>-85451.89</v>
+        <v>-84696.63</v>
       </c>
       <c r="S60" s="84" t="n">
         <v>-0</v>
@@ -5507,7 +5507,7 @@
         <v>0</v>
       </c>
       <c r="R61" s="91" t="n">
-        <v>-84912.10000000001</v>
+        <v>-84156.84000000001</v>
       </c>
       <c r="S61" s="84" t="n">
         <v>-376764.44</v>
@@ -5563,7 +5563,7 @@
         <v>477.18</v>
       </c>
       <c r="M62" s="81" t="n">
-        <v>0.004410437636956255</v>
+        <v>0.004557786755774007</v>
       </c>
       <c r="N62" s="90" t="n">
         <v>0.05500165812722302</v>
@@ -5580,7 +5580,7 @@
         <v>477.18</v>
       </c>
       <c r="R62" s="91" t="n">
-        <v>-84912.10000000001</v>
+        <v>-84156.84000000001</v>
       </c>
       <c r="S62" s="84" t="n">
         <v>-2840048.7</v>
@@ -5592,7 +5592,7 @@
         <v>104695.5519354839</v>
       </c>
       <c r="V62" s="91" t="n">
-        <v>-434.8882511153035</v>
+        <v>-445.8612851428762</v>
       </c>
       <c r="W62" s="75" t="n"/>
     </row>
@@ -5653,7 +5653,7 @@
         <v>417.52</v>
       </c>
       <c r="R63" s="91" t="n">
-        <v>-84912.10000000001</v>
+        <v>-84156.84000000001</v>
       </c>
       <c r="S63" s="84" t="n">
         <v>-2947660.11</v>
@@ -5665,7 +5665,7 @@
         <v>94668.28999999999</v>
       </c>
       <c r="V63" s="91" t="n">
-        <v>-374.491817608628</v>
+        <v>-371.1608590035871</v>
       </c>
       <c r="W63" s="75" t="n"/>
     </row>
@@ -5709,7 +5709,7 @@
         <v>433.37</v>
       </c>
       <c r="M64" s="81" t="n">
-        <v>0.004410327272577286</v>
+        <v>0.004557672695852277</v>
       </c>
       <c r="N64" s="90" t="n">
         <v>0.05500024772757151</v>
@@ -5726,7 +5726,7 @@
         <v>433.37</v>
       </c>
       <c r="R64" s="91" t="n">
-        <v>-84912.10000000001</v>
+        <v>-84156.84000000001</v>
       </c>
       <c r="S64" s="84" t="n">
         <v>-1814864.42</v>
@@ -5738,7 +5738,7 @@
         <v>95085.81</v>
       </c>
       <c r="V64" s="91" t="n">
-        <v>-387.0015597174782</v>
+        <v>-396.3747056021743</v>
       </c>
       <c r="W64" s="75" t="n"/>
     </row>
@@ -5796,10 +5796,10 @@
         <v>0</v>
       </c>
       <c r="Q65" s="83" t="n">
-        <v>0</v>
+        <v>255.9</v>
       </c>
       <c r="R65" s="91" t="n">
-        <v>-85168</v>
+        <v>-84156.84000000001</v>
       </c>
       <c r="S65" s="84" t="n">
         <v>-0</v>
@@ -5869,10 +5869,10 @@
         <v>0</v>
       </c>
       <c r="Q66" s="83" t="n">
-        <v>0</v>
+        <v>74.29000000000001</v>
       </c>
       <c r="R66" s="91" t="n">
-        <v>-85242.28999999999</v>
+        <v>-84156.84000000001</v>
       </c>
       <c r="S66" s="84" t="n">
         <v>-0</v>
@@ -5945,7 +5945,7 @@
         <v>0</v>
       </c>
       <c r="R67" s="91" t="n">
-        <v>-85243.25999999999</v>
+        <v>-84157.81000000001</v>
       </c>
       <c r="S67" s="84" t="n">
         <v>-0</v>
@@ -6018,7 +6018,7 @@
         <v>0</v>
       </c>
       <c r="R68" s="91" t="n">
-        <v>-85243.53999999999</v>
+        <v>-84158.09000000001</v>
       </c>
       <c r="S68" s="84" t="n">
         <v>-0</v>
@@ -6091,7 +6091,7 @@
         <v>0</v>
       </c>
       <c r="R69" s="91" t="n">
-        <v>-85242.56999999999</v>
+        <v>-84157.12000000001</v>
       </c>
       <c r="S69" s="84" t="n">
         <v>-0</v>
@@ -6164,7 +6164,7 @@
         <v>0</v>
       </c>
       <c r="R70" s="91" t="n">
-        <v>-85242.28999999999</v>
+        <v>-84156.84000000001</v>
       </c>
       <c r="S70" s="84" t="n">
         <v>-1150192.44</v>
@@ -6220,7 +6220,7 @@
         <v>435.92</v>
       </c>
       <c r="M71" s="81" t="n">
-        <v>0.004410249379017683</v>
+        <v>0.004557592194033067</v>
       </c>
       <c r="N71" s="90" t="n">
         <v>0.05499925228922997</v>
@@ -6237,7 +6237,7 @@
         <v>435.92</v>
       </c>
       <c r="R71" s="91" t="n">
-        <v>-85242.28999999999</v>
+        <v>-84156.84000000001</v>
       </c>
       <c r="S71" s="84" t="n">
         <v>-2888558.7</v>
@@ -6249,7 +6249,7 @@
         <v>95646.99548387097</v>
       </c>
       <c r="V71" s="91" t="n">
-        <v>-387.577254990522</v>
+        <v>-396.3677039362893</v>
       </c>
       <c r="W71" s="75" t="n"/>
     </row>
@@ -6310,7 +6310,7 @@
         <v>424.65</v>
       </c>
       <c r="R72" s="91" t="n">
-        <v>-85242.28999999999</v>
+        <v>-84156.84000000001</v>
       </c>
       <c r="S72" s="84" t="n">
         <v>-2998008.14</v>
@@ -6322,7 +6322,7 @@
         <v>96285.28999999999</v>
       </c>
       <c r="V72" s="91" t="n">
-        <v>-375.9467146902618</v>
+        <v>-371.15952089877</v>
       </c>
       <c r="W72" s="75" t="n"/>
     </row>
@@ -6366,7 +6366,7 @@
         <v>440.77</v>
       </c>
       <c r="M73" s="81" t="n">
-        <v>0.004410304731360393</v>
+        <v>0.004557649399844488</v>
       </c>
       <c r="N73" s="90" t="n">
         <v>0.05499995966269666</v>
@@ -6383,7 +6383,7 @@
         <v>440.77</v>
       </c>
       <c r="R73" s="91" t="n">
-        <v>-85242.28999999999</v>
+        <v>-84156.84000000001</v>
       </c>
       <c r="S73" s="84" t="n">
         <v>-2914521.3</v>
@@ -6395,7 +6395,7 @@
         <v>96709.94</v>
       </c>
       <c r="V73" s="91" t="n">
-        <v>-388.5044718598697</v>
+        <v>-396.3726794260544</v>
       </c>
       <c r="W73" s="75" t="n"/>
     </row>
@@ -6456,7 +6456,7 @@
         <v>428.46</v>
       </c>
       <c r="R74" s="91" t="n">
-        <v>-85242.28999999999</v>
+        <v>-84156.84000000001</v>
       </c>
       <c r="S74" s="84" t="n">
         <v>-3024954.27</v>
@@ -6468,7 +6468,7 @@
         <v>97150.71000000001</v>
       </c>
       <c r="V74" s="91" t="n">
-        <v>-375.9407581622424</v>
+        <v>-371.1536402194092</v>
       </c>
       <c r="W74" s="75" t="n"/>
     </row>
@@ -6512,7 +6512,7 @@
         <v>444.73</v>
       </c>
       <c r="M75" s="81" t="n">
-        <v>0.004410288413628116</v>
+        <v>0.004557632535714395</v>
       </c>
       <c r="N75" s="90" t="n">
         <v>0.05515451658257575</v>
@@ -6529,7 +6529,7 @@
         <v>444.73</v>
       </c>
       <c r="R75" s="91" t="n">
-        <v>-85242.28999999999</v>
+        <v>-84156.84000000001</v>
       </c>
       <c r="S75" s="84" t="n">
         <v>-3038740.9</v>
@@ -6541,7 +6541,7 @@
         <v>97579.17</v>
       </c>
       <c r="V75" s="91" t="n">
-        <v>-388.5030343228018</v>
+        <v>-396.3712126641124</v>
       </c>
       <c r="W75" s="75" t="n"/>
     </row>
@@ -6585,7 +6585,7 @@
         <v>445.54</v>
       </c>
       <c r="M76" s="81" t="n">
-        <v>0.004398276158800174</v>
+        <v>0.004545218053964462</v>
       </c>
       <c r="N76" s="90" t="n">
         <v>0.05500057349558163</v>
@@ -6602,7 +6602,7 @@
         <v>445.54</v>
       </c>
       <c r="R76" s="91" t="n">
-        <v>-85242.28999999999</v>
+        <v>-84156.84000000001</v>
       </c>
       <c r="S76" s="84" t="n">
         <v>-2855613.76</v>
@@ -6614,7 +6614,7 @@
         <v>98023.89999999999</v>
       </c>
       <c r="V76" s="91" t="n">
-        <v>-387.4447954692743</v>
+        <v>-395.2914602282764</v>
       </c>
       <c r="W76" s="75" t="n"/>
     </row>
@@ -6658,7 +6658,7 @@
         <v>418.62</v>
       </c>
       <c r="M77" s="81" t="n">
-        <v>0.004398185579549407</v>
+        <v>0.004251268210726078</v>
       </c>
       <c r="N77" s="90" t="n">
         <v>0.05499941275525555</v>
@@ -6675,7 +6675,7 @@
         <v>418.62</v>
       </c>
       <c r="R77" s="91" t="n">
-        <v>-85242.28999999999</v>
+        <v>-84156.84000000001</v>
       </c>
       <c r="S77" s="84" t="n">
         <v>-3065529.86</v>
@@ -6687,7 +6687,7 @@
         <v>98469.44</v>
       </c>
       <c r="V77" s="91" t="n">
-        <v>-362.3878376864934</v>
+        <v>-345.8230529497143</v>
       </c>
       <c r="W77" s="75" t="n"/>
     </row>
@@ -6731,7 +6731,7 @@
         <v>449.46</v>
       </c>
       <c r="M78" s="81" t="n">
-        <v>0.00439819988004686</v>
+        <v>0.004545139221054484</v>
       </c>
       <c r="N78" s="90" t="n">
         <v>0.05499959601087667</v>
@@ -6748,7 +6748,7 @@
         <v>449.46</v>
       </c>
       <c r="R78" s="91" t="n">
-        <v>-85242.28999999999</v>
+        <v>-84156.84000000001</v>
       </c>
       <c r="S78" s="84" t="n">
         <v>-2980125.6</v>
@@ -6760,7 +6760,7 @@
         <v>98888.06</v>
       </c>
       <c r="V78" s="91" t="n">
-        <v>-387.4380755715193</v>
+        <v>-395.2846037190311</v>
       </c>
       <c r="W78" s="75" t="n"/>
     </row>
@@ -6821,7 +6821,7 @@
         <v>436.91</v>
       </c>
       <c r="R79" s="91" t="n">
-        <v>-85242.28999999999</v>
+        <v>-84156.84000000001</v>
       </c>
       <c r="S79" s="84" t="n">
         <v>-1596390.88</v>
@@ -6833,7 +6833,7 @@
         <v>99337.52</v>
       </c>
       <c r="V79" s="91" t="n">
-        <v>-374.9158316404446</v>
+        <v>-370.1417648074898</v>
       </c>
       <c r="W79" s="75" t="n"/>
     </row>
@@ -6877,7 +6877,7 @@
         <v>233.8</v>
       </c>
       <c r="M80" s="81" t="n">
-        <v>0.004398164667303472</v>
+        <v>0.004545102829229819</v>
       </c>
       <c r="N80" s="90" t="n">
         <v>0.05499914477255552</v>
@@ -6888,13 +6888,13 @@
         </is>
       </c>
       <c r="P80" s="88" t="n">
-        <v>-13705.39765423249</v>
+        <v>-13802.61077079124</v>
       </c>
       <c r="Q80" s="83" t="n">
         <v>233.8</v>
       </c>
       <c r="R80" s="91" t="n">
-        <v>-71536.8923457675</v>
+        <v>-70354.22922920878</v>
       </c>
       <c r="S80" s="84" t="n">
         <v>-0</v>
@@ -6906,7 +6906,7 @@
         <v>99774.42999999999</v>
       </c>
       <c r="V80" s="91" t="n">
-        <v>-199.7470434258513</v>
+        <v>-203.7849271649868</v>
       </c>
       <c r="W80" s="75" t="n"/>
     </row>
@@ -6967,7 +6967,7 @@
         <v>0</v>
       </c>
       <c r="R81" s="91" t="n">
-        <v>28471.3376542325</v>
+        <v>29654.00077079122</v>
       </c>
       <c r="S81" s="84" t="n">
         <v>0</v>
@@ -7040,7 +7040,7 @@
         <v>0</v>
       </c>
       <c r="R82" s="91" t="n">
-        <v>-71536.8923457675</v>
+        <v>-70354.22922920878</v>
       </c>
       <c r="S82" s="84" t="n">
         <v>-1500123.45</v>
@@ -7096,7 +7096,7 @@
         <v>219.69</v>
       </c>
       <c r="M83" s="81" t="n">
-        <v>0.004398263995305518</v>
+        <v>0.004545205483181158</v>
       </c>
       <c r="N83" s="90" t="n">
         <v>0.05500041762472985</v>
@@ -7113,7 +7113,7 @@
         <v>219.69</v>
       </c>
       <c r="R83" s="91" t="n">
-        <v>-71536.8923457675</v>
+        <v>-70354.22922920878</v>
       </c>
       <c r="S83" s="84" t="n">
         <v>-3006837.6</v>
@@ -7186,7 +7186,7 @@
         <v>440.83</v>
       </c>
       <c r="R84" s="91" t="n">
-        <v>-71536.8923457675</v>
+        <v>-70354.22922920878</v>
       </c>
       <c r="S84" s="84" t="n">
         <v>-3120731.25</v>
@@ -7242,7 +7242,7 @@
         <v>457.56</v>
       </c>
       <c r="M85" s="81" t="n">
-        <v>0.0043982625104384</v>
+        <v>0.004545203948593812</v>
       </c>
       <c r="N85" s="90" t="n">
         <v>0.05500039859668648</v>
@@ -7259,7 +7259,7 @@
         <v>457.56</v>
       </c>
       <c r="R85" s="91" t="n">
-        <v>-71536.8923457675</v>
+        <v>-70354.22922920878</v>
       </c>
       <c r="S85" s="84" t="n">
         <v>-1719147.27</v>
@@ -7329,10 +7329,10 @@
         <v>0</v>
       </c>
       <c r="Q86" s="83" t="n">
-        <v>0</v>
+        <v>255.9</v>
       </c>
       <c r="R86" s="91" t="n">
-        <v>-71792.79234576749</v>
+        <v>-70354.22922920878</v>
       </c>
       <c r="S86" s="84" t="n">
         <v>-0</v>
@@ -7402,10 +7402,10 @@
         <v>0</v>
       </c>
       <c r="Q87" s="83" t="n">
-        <v>0</v>
+        <v>74.29000000000001</v>
       </c>
       <c r="R87" s="91" t="n">
-        <v>-71867.08234576749</v>
+        <v>-70354.22922920878</v>
       </c>
       <c r="S87" s="84" t="n">
         <v>-1420391</v>
@@ -7461,7 +7461,7 @@
         <v>460.31</v>
       </c>
       <c r="M88" s="81" t="n">
-        <v>0.00439819108808015</v>
+        <v>0.004545130134693265</v>
       </c>
       <c r="N88" s="90" t="n">
         <v>0.05499948334505067</v>
@@ -7478,7 +7478,7 @@
         <v>460.31</v>
       </c>
       <c r="R88" s="91" t="n">
-        <v>-71867.08234576749</v>
+        <v>-70354.22922920878</v>
       </c>
       <c r="S88" s="84" t="n">
         <v>-3057504.3</v>
@@ -7551,7 +7551,7 @@
         <v>448.25</v>
       </c>
       <c r="R89" s="91" t="n">
-        <v>-71867.08234576749</v>
+        <v>-70354.22922920878</v>
       </c>
       <c r="S89" s="84" t="n">
         <v>-3173316.86</v>
@@ -7607,7 +7607,7 @@
         <v>465.27</v>
       </c>
       <c r="M90" s="81" t="n">
-        <v>0.00439826180235503</v>
+        <v>0.004545203216800742</v>
       </c>
       <c r="N90" s="90" t="n">
         <v>0.05500038952285258</v>
@@ -7624,7 +7624,7 @@
         <v>465.27</v>
       </c>
       <c r="R90" s="91" t="n">
-        <v>-71867.08234576749</v>
+        <v>-70354.22922920878</v>
       </c>
       <c r="S90" s="84" t="n">
         <v>-3084909.9</v>
@@ -7697,7 +7697,7 @@
         <v>452.27</v>
       </c>
       <c r="R91" s="91" t="n">
-        <v>-71867.08234576749</v>
+        <v>-70354.22922920878</v>
       </c>
       <c r="S91" s="84" t="n">
         <v>-3201760.6</v>
@@ -7753,7 +7753,7 @@
         <v>469.44</v>
       </c>
       <c r="M92" s="81" t="n">
-        <v>0.004398258001007127</v>
+        <v>0.004545199288166657</v>
       </c>
       <c r="N92" s="90" t="n">
         <v>0.05484601912472131</v>
@@ -7770,7 +7770,7 @@
         <v>469.44</v>
       </c>
       <c r="R92" s="91" t="n">
-        <v>-71867.08234576749</v>
+        <v>-70354.22922920878</v>
       </c>
       <c r="S92" s="84" t="n">
         <v>-3216313.24</v>
@@ -7826,7 +7826,7 @@
         <v>472.87</v>
       </c>
       <c r="M93" s="81" t="n">
-        <v>0.004410347418340788</v>
+        <v>0.00455769351619506</v>
       </c>
       <c r="N93" s="90" t="n">
         <v>0.05500050517987431</v>
@@ -7843,7 +7843,7 @@
         <v>472.87</v>
       </c>
       <c r="R93" s="91" t="n">
-        <v>-71867.08234576749</v>
+        <v>-70354.22922920878</v>
       </c>
       <c r="S93" s="84" t="n">
         <v>-312674.73</v>
@@ -7902,7 +7902,7 @@
         <v>0.0008333382603676356</v>
       </c>
       <c r="N94" s="90" t="n">
-        <v>0.009373418609034623</v>
+        <v>0.01019037987659588</v>
       </c>
       <c r="O94" s="82" t="inlineStr">
         <is>
@@ -7913,10 +7913,10 @@
         <v>0</v>
       </c>
       <c r="Q94" s="83" t="n">
-        <v>0</v>
+        <v>730.62</v>
       </c>
       <c r="R94" s="91" t="n">
-        <v>-72597.70234576748</v>
+        <v>-70354.22922920878</v>
       </c>
       <c r="S94" s="84" t="n">
         <v>-0</v>
@@ -7972,7 +7972,7 @@
         <v>45.88</v>
       </c>
       <c r="M95" s="81" t="n">
-        <v>0.004410748912710316</v>
+        <v>0.004116094674724957</v>
       </c>
       <c r="N95" s="90" t="n">
         <v>0.0550056360796074</v>
@@ -7989,7 +7989,7 @@
         <v>45.88</v>
       </c>
       <c r="R95" s="91" t="n">
-        <v>-72597.70234576748</v>
+        <v>-70354.22922920878</v>
       </c>
       <c r="S95" s="84" t="n">
         <v>-0</v>
@@ -8062,7 +8062,7 @@
         <v>0</v>
       </c>
       <c r="R96" s="91" t="n">
-        <v>-74697.73234576748</v>
+        <v>-72454.25922920878</v>
       </c>
       <c r="S96" s="84" t="n">
         <v>-0</v>

</xml_diff>

<commit_message>
ajustando arquivos docx e os preenchimento
</commit_message>
<xml_diff>
--- a/relatorio_final.xlsx
+++ b/relatorio_final.xlsx
@@ -1396,9 +1396,10 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="135">
-        <f>"Recálculo da operação nº "&amp;AA1&amp;" - Capitalização "&amp;AA2</f>
-        <v/>
+      <c r="A1" s="135" t="inlineStr">
+        <is>
+          <t>Recálculo da operação nº 156.894.779-10 - Capitalização Afastada</t>
+        </is>
       </c>
       <c r="B1" s="30" t="n"/>
       <c r="C1" s="31" t="n"/>
@@ -1519,9 +1520,8 @@
           <t>Valor Liberado:</t>
         </is>
       </c>
-      <c r="B3" s="44">
-        <f>SUMIF($B$13:$B$19,#REF!,$C$13:$C$19)</f>
-        <v/>
+      <c r="B3" s="44" t="n">
+        <v>15000</v>
       </c>
       <c r="C3" s="137" t="inlineStr">
         <is>
@@ -7913,10 +7913,10 @@
         <v>0</v>
       </c>
       <c r="Q94" s="83" t="n">
-        <v>730.62</v>
+        <v>0</v>
       </c>
       <c r="R94" s="91" t="n">
-        <v>-70354.22922920878</v>
+        <v>-71084.84922920878</v>
       </c>
       <c r="S94" s="84" t="n">
         <v>-0</v>
@@ -7989,7 +7989,7 @@
         <v>45.88</v>
       </c>
       <c r="R95" s="91" t="n">
-        <v>-70354.22922920878</v>
+        <v>-71084.84922920878</v>
       </c>
       <c r="S95" s="84" t="n">
         <v>-0</v>
@@ -8062,7 +8062,7 @@
         <v>0</v>
       </c>
       <c r="R96" s="91" t="n">
-        <v>-72454.25922920878</v>
+        <v>-73184.87922920877</v>
       </c>
       <c r="S96" s="84" t="n">
         <v>-0</v>

</xml_diff>

<commit_message>
corrigingo nos if no laudo_completo.docx
</commit_message>
<xml_diff>
--- a/relatorio_final.xlsx
+++ b/relatorio_final.xlsx
@@ -1398,7 +1398,7 @@
     <row r="1">
       <c r="A1" s="135" t="inlineStr">
         <is>
-          <t>Recálculo da operação nº 156.894.779-10 - Capitalização Afastada</t>
+          <t>Recálculo da operação nº 159.789.999-10 - Capitalização Afastada</t>
         </is>
       </c>
       <c r="B1" s="30" t="n"/>
@@ -1521,7 +1521,7 @@
         </is>
       </c>
       <c r="B3" s="44" t="n">
-        <v>15000</v>
+        <v>120000</v>
       </c>
       <c r="C3" s="137" t="inlineStr">
         <is>
@@ -7913,10 +7913,10 @@
         <v>0</v>
       </c>
       <c r="Q94" s="83" t="n">
-        <v>0</v>
+        <v>730.62</v>
       </c>
       <c r="R94" s="91" t="n">
-        <v>-71084.84922920878</v>
+        <v>-70354.22922920878</v>
       </c>
       <c r="S94" s="84" t="n">
         <v>-0</v>
@@ -7989,7 +7989,7 @@
         <v>45.88</v>
       </c>
       <c r="R95" s="91" t="n">
-        <v>-71084.84922920878</v>
+        <v>-70354.22922920878</v>
       </c>
       <c r="S95" s="84" t="n">
         <v>-0</v>
@@ -8062,7 +8062,7 @@
         <v>0</v>
       </c>
       <c r="R96" s="91" t="n">
-        <v>-73184.87922920877</v>
+        <v>-72454.25922920878</v>
       </c>
       <c r="S96" s="84" t="n">
         <v>-0</v>

</xml_diff>

<commit_message>
corrigindo os formatos nos laudos
</commit_message>
<xml_diff>
--- a/relatorio_final.xlsx
+++ b/relatorio_final.xlsx
@@ -1398,7 +1398,7 @@
     <row r="1">
       <c r="A1" s="135" t="inlineStr">
         <is>
-          <t>Recálculo da operação nº 159.789.999-10 - Capitalização Afastada</t>
+          <t>Recálculo da operação nº 145.789.000-10 - Capitalização Afastada</t>
         </is>
       </c>
       <c r="B1" s="30" t="n"/>
@@ -1521,7 +1521,7 @@
         </is>
       </c>
       <c r="B3" s="44" t="n">
-        <v>120000</v>
+        <v>80000</v>
       </c>
       <c r="C3" s="137" t="inlineStr">
         <is>
@@ -1578,7 +1578,7 @@
         </is>
       </c>
       <c r="D4" s="49" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E4" s="50" t="inlineStr">
         <is>
@@ -2511,10 +2511,10 @@
         <v>0</v>
       </c>
       <c r="Q20" s="83" t="n">
-        <v>305.66</v>
+        <v>0</v>
       </c>
       <c r="R20" s="91" t="n">
-        <v>-56241.5</v>
+        <v>-56547.16</v>
       </c>
       <c r="S20" s="84" t="n">
         <v>-0</v>
@@ -2584,10 +2584,10 @@
         <v>0</v>
       </c>
       <c r="Q21" s="83" t="n">
-        <v>88.73999999999999</v>
+        <v>0</v>
       </c>
       <c r="R21" s="91" t="n">
-        <v>-56241.5</v>
+        <v>-56635.9</v>
       </c>
       <c r="S21" s="84" t="n">
         <v>-0</v>
@@ -2660,7 +2660,7 @@
         <v>0</v>
       </c>
       <c r="R22" s="91" t="n">
-        <v>-56242.66</v>
+        <v>-56637.06</v>
       </c>
       <c r="S22" s="84" t="n">
         <v>-0</v>
@@ -2733,7 +2733,7 @@
         <v>0</v>
       </c>
       <c r="R23" s="91" t="n">
-        <v>-56243</v>
+        <v>-56637.4</v>
       </c>
       <c r="S23" s="84" t="n">
         <v>-0</v>
@@ -2806,7 +2806,7 @@
         <v>0</v>
       </c>
       <c r="R24" s="91" t="n">
-        <v>-56241.84</v>
+        <v>-56636.24</v>
       </c>
       <c r="S24" s="84" t="n">
         <v>-0</v>
@@ -2879,7 +2879,7 @@
         <v>0</v>
       </c>
       <c r="R25" s="91" t="n">
-        <v>-56241.5</v>
+        <v>-56635.9</v>
       </c>
       <c r="S25" s="84" t="n">
         <v>-0</v>
@@ -2952,7 +2952,7 @@
         <v>0</v>
       </c>
       <c r="R26" s="91" t="n">
-        <v>-96241.5</v>
+        <v>-96635.89999999999</v>
       </c>
       <c r="S26" s="84" t="n">
         <v>-0</v>
@@ -3025,7 +3025,7 @@
         <v>0</v>
       </c>
       <c r="R27" s="91" t="n">
-        <v>-96393.5</v>
+        <v>-96787.89999999999</v>
       </c>
       <c r="S27" s="84" t="n">
         <v>-0</v>
@@ -3098,7 +3098,7 @@
         <v>0</v>
       </c>
       <c r="R28" s="91" t="n">
-        <v>-96241.5</v>
+        <v>-96635.89999999999</v>
       </c>
       <c r="S28" s="84" t="n">
         <v>-1546174.4</v>
@@ -3171,7 +3171,7 @@
         <v>243.61</v>
       </c>
       <c r="R29" s="91" t="n">
-        <v>-96241.5</v>
+        <v>-96635.89999999999</v>
       </c>
       <c r="S29" s="84" t="n">
         <v>-2906385.3</v>
@@ -3183,7 +3183,7 @@
         <v>92147.63333333333</v>
       </c>
       <c r="V29" s="91" t="n">
-        <v>-250.7836595524696</v>
+        <v>-251.7414155233643</v>
       </c>
       <c r="W29" s="75" t="n"/>
     </row>
@@ -3244,7 +3244,7 @@
         <v>427.27</v>
       </c>
       <c r="R30" s="91" t="n">
-        <v>-96241.5</v>
+        <v>-96635.89999999999</v>
       </c>
       <c r="S30" s="84" t="n">
         <v>-3016510.18</v>
@@ -3256,7 +3256,7 @@
         <v>96879.50999999999</v>
       </c>
       <c r="V30" s="91" t="n">
-        <v>-424.4561693695529</v>
+        <v>-426.1956010409145</v>
       </c>
       <c r="W30" s="75" t="n"/>
     </row>
@@ -3317,7 +3317,7 @@
         <v>443.49</v>
       </c>
       <c r="R31" s="91" t="n">
-        <v>-96241.5</v>
+        <v>-96635.89999999999</v>
       </c>
       <c r="S31" s="84" t="n">
         <v>-2932508.1</v>
@@ -3329,7 +3329,7 @@
         <v>97306.78</v>
       </c>
       <c r="V31" s="91" t="n">
-        <v>-453.2903695103708</v>
+        <v>-455.1479644328822</v>
       </c>
       <c r="W31" s="75" t="n"/>
     </row>
@@ -3390,7 +3390,7 @@
         <v>431.11</v>
       </c>
       <c r="R32" s="91" t="n">
-        <v>-96241.5</v>
+        <v>-96635.89999999999</v>
       </c>
       <c r="S32" s="84" t="n">
         <v>-3043622.78</v>
@@ -3402,7 +3402,7 @@
         <v>97750.27</v>
       </c>
       <c r="V32" s="91" t="n">
-        <v>-424.4558410426828</v>
+        <v>-426.1952713685529</v>
       </c>
       <c r="W32" s="75" t="n"/>
     </row>
@@ -3463,7 +3463,7 @@
         <v>447.48</v>
       </c>
       <c r="R33" s="91" t="n">
-        <v>-96241.5</v>
+        <v>-96635.89999999999</v>
       </c>
       <c r="S33" s="84" t="n">
         <v>-3057494.66</v>
@@ -3475,7 +3475,7 @@
         <v>98181.38</v>
       </c>
       <c r="V33" s="91" t="n">
-        <v>-453.2943017623195</v>
+        <v>-455.1519127992948</v>
       </c>
       <c r="W33" s="75" t="n"/>
     </row>
@@ -3536,7 +3536,7 @@
         <v>449.52</v>
       </c>
       <c r="R34" s="91" t="n">
-        <v>-96241.5</v>
+        <v>-96635.89999999999</v>
       </c>
       <c r="S34" s="84" t="n">
         <v>-2774194.64</v>
@@ -3548,7 +3548,7 @@
         <v>98628.86</v>
       </c>
       <c r="V34" s="91" t="n">
-        <v>-453.2948324393108</v>
+        <v>-455.1524456510132</v>
       </c>
       <c r="W34" s="75" t="n"/>
     </row>
@@ -3609,7 +3609,7 @@
         <v>407.78</v>
       </c>
       <c r="R35" s="91" t="n">
-        <v>-96241.5</v>
+        <v>-96635.89999999999</v>
       </c>
       <c r="S35" s="84" t="n">
         <v>-3084070.96</v>
@@ -3621,7 +3621,7 @@
         <v>99078.38</v>
       </c>
       <c r="V35" s="91" t="n">
-        <v>-369.6465745505615</v>
+        <v>-371.16139517371</v>
       </c>
       <c r="W35" s="75" t="n"/>
     </row>
@@ -3682,7 +3682,7 @@
         <v>453.42</v>
       </c>
       <c r="R36" s="91" t="n">
-        <v>-96241.5</v>
+        <v>-96635.89999999999</v>
       </c>
       <c r="S36" s="84" t="n">
         <v>-2998187.4</v>
@@ -3694,7 +3694,7 @@
         <v>99486.16</v>
       </c>
       <c r="V36" s="91" t="n">
-        <v>-453.2875243760486</v>
+        <v>-455.1451076391307</v>
       </c>
       <c r="W36" s="75" t="n"/>
     </row>
@@ -3755,7 +3755,7 @@
         <v>440.76</v>
       </c>
       <c r="R37" s="91" t="n">
-        <v>-96241.5</v>
+        <v>-96635.89999999999</v>
       </c>
       <c r="S37" s="84" t="n">
         <v>-3111790.54</v>
@@ -3767,7 +3767,7 @@
         <v>99939.58</v>
       </c>
       <c r="V37" s="91" t="n">
-        <v>-424.4504883850855</v>
+        <v>-426.1898967756351</v>
       </c>
       <c r="W37" s="75" t="n"/>
     </row>
@@ -3828,7 +3828,7 @@
         <v>457.5</v>
       </c>
       <c r="R38" s="91" t="n">
-        <v>-96241.5</v>
+        <v>-96635.89999999999</v>
       </c>
       <c r="S38" s="84" t="n">
         <v>-3025135.2</v>
@@ -3840,7 +3840,7 @@
         <v>100380.34</v>
       </c>
       <c r="V38" s="91" t="n">
-        <v>-453.2921501490778</v>
+        <v>-455.1497523686898</v>
       </c>
       <c r="W38" s="75" t="n"/>
     </row>
@@ -3901,7 +3901,7 @@
         <v>444.73</v>
       </c>
       <c r="R39" s="91" t="n">
-        <v>-96241.5</v>
+        <v>-96635.89999999999</v>
       </c>
       <c r="S39" s="84" t="n">
         <v>-3139759.67</v>
@@ -3913,7 +3913,7 @@
         <v>100837.84</v>
       </c>
       <c r="V39" s="91" t="n">
-        <v>-424.4585395224573</v>
+        <v>-426.197980906763</v>
       </c>
       <c r="W39" s="75" t="n"/>
     </row>
@@ -3974,7 +3974,7 @@
         <v>461.61</v>
       </c>
       <c r="R40" s="91" t="n">
-        <v>-96241.5</v>
+        <v>-96635.89999999999</v>
       </c>
       <c r="S40" s="84" t="n">
         <v>-2034883.6</v>
@@ -3986,7 +3986,7 @@
         <v>101282.57</v>
       </c>
       <c r="V40" s="91" t="n">
-        <v>-453.2901247364134</v>
+        <v>-455.1477186558352</v>
       </c>
       <c r="W40" s="75" t="n"/>
     </row>
@@ -4044,10 +4044,10 @@
         <v>0</v>
       </c>
       <c r="Q41" s="83" t="n">
-        <v>279.67</v>
+        <v>0</v>
       </c>
       <c r="R41" s="91" t="n">
-        <v>-96241.5</v>
+        <v>-96915.56999999999</v>
       </c>
       <c r="S41" s="84" t="n">
         <v>-0</v>
@@ -4117,10 +4117,10 @@
         <v>0</v>
       </c>
       <c r="Q42" s="83" t="n">
-        <v>81.19</v>
+        <v>0</v>
       </c>
       <c r="R42" s="91" t="n">
-        <v>-96241.5</v>
+        <v>-96996.75999999999</v>
       </c>
       <c r="S42" s="84" t="n">
         <v>-0</v>
@@ -4193,7 +4193,7 @@
         <v>0</v>
       </c>
       <c r="R43" s="91" t="n">
-        <v>-96242.56</v>
+        <v>-96997.81999999999</v>
       </c>
       <c r="S43" s="84" t="n">
         <v>-0</v>
@@ -4266,7 +4266,7 @@
         <v>0</v>
       </c>
       <c r="R44" s="91" t="n">
-        <v>-96242.87</v>
+        <v>-96998.12999999999</v>
       </c>
       <c r="S44" s="84" t="n">
         <v>-0</v>
@@ -4339,7 +4339,7 @@
         <v>0</v>
       </c>
       <c r="R45" s="91" t="n">
-        <v>-96241.81</v>
+        <v>-96997.06999999999</v>
       </c>
       <c r="S45" s="84" t="n">
         <v>-0</v>
@@ -4412,7 +4412,7 @@
         <v>0</v>
       </c>
       <c r="R46" s="91" t="n">
-        <v>-96241.5</v>
+        <v>-96996.75999999999</v>
       </c>
       <c r="S46" s="84" t="n">
         <v>-1123155.44</v>
@@ -4485,7 +4485,7 @@
         <v>464.3</v>
       </c>
       <c r="R47" s="91" t="n">
-        <v>-96241.5</v>
+        <v>-96996.75999999999</v>
       </c>
       <c r="S47" s="84" t="n">
         <v>-3077080.2</v>
@@ -4497,7 +4497,7 @@
         <v>101872.2270967742</v>
       </c>
       <c r="V47" s="91" t="n">
-        <v>-453.2926166909854</v>
+        <v>-455.7533161977407</v>
       </c>
       <c r="W47" s="75" t="n"/>
     </row>
@@ -4558,7 +4558,7 @@
         <v>452.36</v>
       </c>
       <c r="R48" s="91" t="n">
-        <v>-96241.5</v>
+        <v>-96996.75999999999</v>
       </c>
       <c r="S48" s="84" t="n">
         <v>-3193672.7</v>
@@ -4570,7 +4570,7 @@
         <v>102569.34</v>
       </c>
       <c r="V48" s="91" t="n">
-        <v>-424.4524235019908</v>
+        <v>-427.7833351915854</v>
       </c>
       <c r="W48" s="75" t="n"/>
     </row>
@@ -4631,7 +4631,7 @@
         <v>469.54</v>
       </c>
       <c r="R49" s="91" t="n">
-        <v>-96241.5</v>
+        <v>-96996.75999999999</v>
       </c>
       <c r="S49" s="84" t="n">
         <v>-3104737.2</v>
@@ -4643,7 +4643,7 @@
         <v>103021.7</v>
       </c>
       <c r="V49" s="91" t="n">
-        <v>-453.2936610979489</v>
+        <v>-456.8509058466366</v>
       </c>
       <c r="W49" s="75" t="n"/>
     </row>
@@ -4704,7 +4704,7 @@
         <v>456.43</v>
       </c>
       <c r="R50" s="91" t="n">
-        <v>-96241.5</v>
+        <v>-96996.75999999999</v>
       </c>
       <c r="S50" s="84" t="n">
         <v>-3222377.77</v>
@@ -4716,7 +4716,7 @@
         <v>103491.24</v>
       </c>
       <c r="V50" s="91" t="n">
-        <v>-424.4562906483631</v>
+        <v>-427.7872326855828</v>
       </c>
       <c r="W50" s="75" t="n"/>
     </row>
@@ -4777,7 +4777,7 @@
         <v>473.76</v>
       </c>
       <c r="R51" s="91" t="n">
-        <v>-96241.5</v>
+        <v>-96996.75999999999</v>
       </c>
       <c r="S51" s="84" t="n">
         <v>-3237064.33</v>
@@ -4789,7 +4789,7 @@
         <v>103947.67</v>
       </c>
       <c r="V51" s="91" t="n">
-        <v>-453.2933975045624</v>
+        <v>-456.8506401846879</v>
       </c>
       <c r="W51" s="75" t="n"/>
     </row>
@@ -4850,7 +4850,7 @@
         <v>475.92</v>
       </c>
       <c r="R52" s="91" t="n">
-        <v>-96241.5</v>
+        <v>-96996.75999999999</v>
       </c>
       <c r="S52" s="84" t="n">
         <v>-2937125.8</v>
@@ -4862,7 +4862,7 @@
         <v>104421.43</v>
       </c>
       <c r="V52" s="91" t="n">
-        <v>-453.2941161989432</v>
+        <v>-456.8513645190588</v>
       </c>
       <c r="W52" s="75" t="n"/>
     </row>
@@ -4923,7 +4923,7 @@
         <v>431.72</v>
       </c>
       <c r="R53" s="91" t="n">
-        <v>-96241.5</v>
+        <v>-96996.75999999999</v>
       </c>
       <c r="S53" s="84" t="n">
         <v>-3265201.17</v>
@@ -4935,7 +4935,7 @@
         <v>104897.35</v>
       </c>
       <c r="V53" s="91" t="n">
-        <v>-369.6385979429375</v>
+        <v>-372.5393553862689</v>
       </c>
       <c r="W53" s="75" t="n"/>
     </row>
@@ -4996,7 +4996,7 @@
         <v>480.05</v>
       </c>
       <c r="R54" s="91" t="n">
-        <v>-96241.5</v>
+        <v>-96996.75999999999</v>
       </c>
       <c r="S54" s="84" t="n">
         <v>-3174273.6</v>
@@ -5008,7 +5008,7 @@
         <v>105329.07</v>
       </c>
       <c r="V54" s="91" t="n">
-        <v>-453.2877539742529</v>
+        <v>-456.8449523664911</v>
       </c>
       <c r="W54" s="75" t="n"/>
     </row>
@@ -5069,7 +5069,7 @@
         <v>466.65</v>
       </c>
       <c r="R55" s="91" t="n">
-        <v>-96241.5</v>
+        <v>-96996.75999999999</v>
       </c>
       <c r="S55" s="84" t="n">
         <v>-1700412.32</v>
@@ -5081,7 +5081,7 @@
         <v>105809.12</v>
       </c>
       <c r="V55" s="91" t="n">
-        <v>-424.4539220721303</v>
+        <v>-427.7848455218292</v>
       </c>
       <c r="W55" s="75" t="n"/>
     </row>
@@ -5142,7 +5142,7 @@
         <v>0</v>
       </c>
       <c r="R56" s="91" t="n">
-        <v>-96182.58</v>
+        <v>-96937.84</v>
       </c>
       <c r="S56" s="84" t="n">
         <v>-1168385.35</v>
@@ -5215,7 +5215,7 @@
         <v>0</v>
       </c>
       <c r="R57" s="91" t="n">
-        <v>-96098.67</v>
+        <v>-96853.92999999999</v>
       </c>
       <c r="S57" s="84" t="n">
         <v>-0</v>
@@ -5288,7 +5288,7 @@
         <v>0</v>
       </c>
       <c r="R58" s="91" t="n">
-        <v>-89849.61</v>
+        <v>-90604.87</v>
       </c>
       <c r="S58" s="84" t="n">
         <v>-0</v>
@@ -5361,7 +5361,7 @@
         <v>0</v>
       </c>
       <c r="R59" s="91" t="n">
-        <v>-89141.07000000001</v>
+        <v>-89896.33</v>
       </c>
       <c r="S59" s="84" t="n">
         <v>-0</v>
@@ -5434,7 +5434,7 @@
         <v>0</v>
       </c>
       <c r="R60" s="91" t="n">
-        <v>-84696.63</v>
+        <v>-85451.89</v>
       </c>
       <c r="S60" s="84" t="n">
         <v>-0</v>
@@ -5507,7 +5507,7 @@
         <v>0</v>
       </c>
       <c r="R61" s="91" t="n">
-        <v>-84156.84000000001</v>
+        <v>-84912.10000000001</v>
       </c>
       <c r="S61" s="84" t="n">
         <v>-376764.44</v>
@@ -5580,7 +5580,7 @@
         <v>477.18</v>
       </c>
       <c r="R62" s="91" t="n">
-        <v>-84156.84000000001</v>
+        <v>-84912.10000000001</v>
       </c>
       <c r="S62" s="84" t="n">
         <v>-2840048.7</v>
@@ -5592,7 +5592,7 @@
         <v>104695.5519354839</v>
       </c>
       <c r="V62" s="91" t="n">
-        <v>-445.8612851428762</v>
+        <v>-449.4186127781232</v>
       </c>
       <c r="W62" s="75" t="n"/>
     </row>
@@ -5653,7 +5653,7 @@
         <v>417.52</v>
       </c>
       <c r="R63" s="91" t="n">
-        <v>-84156.84000000001</v>
+        <v>-84912.10000000001</v>
       </c>
       <c r="S63" s="84" t="n">
         <v>-2947660.11</v>
@@ -5665,7 +5665,7 @@
         <v>94668.28999999999</v>
       </c>
       <c r="V63" s="91" t="n">
-        <v>-371.1608590035871</v>
+        <v>-374.491817608628</v>
       </c>
       <c r="W63" s="75" t="n"/>
     </row>
@@ -5726,7 +5726,7 @@
         <v>433.37</v>
       </c>
       <c r="R64" s="91" t="n">
-        <v>-84156.84000000001</v>
+        <v>-84912.10000000001</v>
       </c>
       <c r="S64" s="84" t="n">
         <v>-1814864.42</v>
@@ -5738,7 +5738,7 @@
         <v>95085.81</v>
       </c>
       <c r="V64" s="91" t="n">
-        <v>-396.3747056021743</v>
+        <v>-399.9319442075342</v>
       </c>
       <c r="W64" s="75" t="n"/>
     </row>
@@ -5796,10 +5796,10 @@
         <v>0</v>
       </c>
       <c r="Q65" s="83" t="n">
-        <v>255.9</v>
+        <v>0</v>
       </c>
       <c r="R65" s="91" t="n">
-        <v>-84156.84000000001</v>
+        <v>-85168</v>
       </c>
       <c r="S65" s="84" t="n">
         <v>-0</v>
@@ -5869,10 +5869,10 @@
         <v>0</v>
       </c>
       <c r="Q66" s="83" t="n">
-        <v>74.29000000000001</v>
+        <v>0</v>
       </c>
       <c r="R66" s="91" t="n">
-        <v>-84156.84000000001</v>
+        <v>-85242.28999999999</v>
       </c>
       <c r="S66" s="84" t="n">
         <v>-0</v>
@@ -5945,7 +5945,7 @@
         <v>0</v>
       </c>
       <c r="R67" s="91" t="n">
-        <v>-84157.81000000001</v>
+        <v>-85243.25999999999</v>
       </c>
       <c r="S67" s="84" t="n">
         <v>-0</v>
@@ -6018,7 +6018,7 @@
         <v>0</v>
       </c>
       <c r="R68" s="91" t="n">
-        <v>-84158.09000000001</v>
+        <v>-85243.53999999999</v>
       </c>
       <c r="S68" s="84" t="n">
         <v>-0</v>
@@ -6091,7 +6091,7 @@
         <v>0</v>
       </c>
       <c r="R69" s="91" t="n">
-        <v>-84157.12000000001</v>
+        <v>-85242.56999999999</v>
       </c>
       <c r="S69" s="84" t="n">
         <v>-0</v>
@@ -6164,7 +6164,7 @@
         <v>0</v>
       </c>
       <c r="R70" s="91" t="n">
-        <v>-84156.84000000001</v>
+        <v>-85242.28999999999</v>
       </c>
       <c r="S70" s="84" t="n">
         <v>-1150192.44</v>
@@ -6237,7 +6237,7 @@
         <v>435.92</v>
       </c>
       <c r="R71" s="91" t="n">
-        <v>-84156.84000000001</v>
+        <v>-85242.28999999999</v>
       </c>
       <c r="S71" s="84" t="n">
         <v>-2888558.7</v>
@@ -6249,7 +6249,7 @@
         <v>95646.99548387097</v>
       </c>
       <c r="V71" s="91" t="n">
-        <v>-396.3677039362893</v>
+        <v>-400.5268739092156</v>
       </c>
       <c r="W71" s="75" t="n"/>
     </row>
@@ -6310,7 +6310,7 @@
         <v>424.65</v>
       </c>
       <c r="R72" s="91" t="n">
-        <v>-84156.84000000001</v>
+        <v>-85242.28999999999</v>
       </c>
       <c r="S72" s="84" t="n">
         <v>-2998008.14</v>
@@ -6322,7 +6322,7 @@
         <v>96285.28999999999</v>
       </c>
       <c r="V72" s="91" t="n">
-        <v>-371.15952089877</v>
+        <v>-375.9467146902618</v>
       </c>
       <c r="W72" s="75" t="n"/>
     </row>
@@ -6383,7 +6383,7 @@
         <v>440.77</v>
       </c>
       <c r="R73" s="91" t="n">
-        <v>-84156.84000000001</v>
+        <v>-85242.28999999999</v>
       </c>
       <c r="S73" s="84" t="n">
         <v>-2914521.3</v>
@@ -6395,7 +6395,7 @@
         <v>96709.94</v>
       </c>
       <c r="V73" s="91" t="n">
-        <v>-396.3726794260544</v>
+        <v>-401.4850710615175</v>
       </c>
       <c r="W73" s="75" t="n"/>
     </row>
@@ -6456,7 +6456,7 @@
         <v>428.46</v>
       </c>
       <c r="R74" s="91" t="n">
-        <v>-84156.84000000001</v>
+        <v>-85242.28999999999</v>
       </c>
       <c r="S74" s="84" t="n">
         <v>-3024954.27</v>
@@ -6468,7 +6468,7 @@
         <v>97150.71000000001</v>
       </c>
       <c r="V74" s="91" t="n">
-        <v>-371.1536402194092</v>
+        <v>-375.9407581622424</v>
       </c>
       <c r="W74" s="75" t="n"/>
     </row>
@@ -6529,7 +6529,7 @@
         <v>444.73</v>
       </c>
       <c r="R75" s="91" t="n">
-        <v>-84156.84000000001</v>
+        <v>-85242.28999999999</v>
       </c>
       <c r="S75" s="84" t="n">
         <v>-3038740.9</v>
@@ -6541,7 +6541,7 @@
         <v>97579.17</v>
       </c>
       <c r="V75" s="91" t="n">
-        <v>-396.3712126641124</v>
+        <v>-401.4835853813657</v>
       </c>
       <c r="W75" s="75" t="n"/>
     </row>
@@ -6602,7 +6602,7 @@
         <v>445.54</v>
       </c>
       <c r="R76" s="91" t="n">
-        <v>-84156.84000000001</v>
+        <v>-85242.28999999999</v>
       </c>
       <c r="S76" s="84" t="n">
         <v>-2855613.76</v>
@@ -6614,7 +6614,7 @@
         <v>98023.89999999999</v>
       </c>
       <c r="V76" s="91" t="n">
-        <v>-395.2914602282764</v>
+        <v>-400.3899063617669</v>
       </c>
       <c r="W76" s="75" t="n"/>
     </row>
@@ -6675,7 +6675,7 @@
         <v>418.62</v>
       </c>
       <c r="R77" s="91" t="n">
-        <v>-84156.84000000001</v>
+        <v>-85242.28999999999</v>
       </c>
       <c r="S77" s="84" t="n">
         <v>-3065529.86</v>
@@ -6687,7 +6687,7 @@
         <v>98469.44</v>
       </c>
       <c r="V77" s="91" t="n">
-        <v>-345.8230529497143</v>
+        <v>-350.2834584595251</v>
       </c>
       <c r="W77" s="75" t="n"/>
     </row>
@@ -6748,7 +6748,7 @@
         <v>449.46</v>
       </c>
       <c r="R78" s="91" t="n">
-        <v>-84156.84000000001</v>
+        <v>-85242.28999999999</v>
       </c>
       <c r="S78" s="84" t="n">
         <v>-2980125.6</v>
@@ -6760,7 +6760,7 @@
         <v>98888.06</v>
       </c>
       <c r="V78" s="91" t="n">
-        <v>-395.2846037190311</v>
+        <v>-400.3829614176663</v>
       </c>
       <c r="W78" s="75" t="n"/>
     </row>
@@ -6821,7 +6821,7 @@
         <v>436.91</v>
       </c>
       <c r="R79" s="91" t="n">
-        <v>-84156.84000000001</v>
+        <v>-85242.28999999999</v>
       </c>
       <c r="S79" s="84" t="n">
         <v>-1596390.88</v>
@@ -6833,7 +6833,7 @@
         <v>99337.52</v>
       </c>
       <c r="V79" s="91" t="n">
-        <v>-370.1417648074898</v>
+        <v>-374.9158316404446</v>
       </c>
       <c r="W79" s="75" t="n"/>
     </row>
@@ -6888,13 +6888,13 @@
         </is>
       </c>
       <c r="P80" s="88" t="n">
-        <v>-13802.61077079124</v>
+        <v>-13909.23327915017</v>
       </c>
       <c r="Q80" s="83" t="n">
         <v>233.8</v>
       </c>
       <c r="R80" s="91" t="n">
-        <v>-70354.22922920878</v>
+        <v>-71333.05672084983</v>
       </c>
       <c r="S80" s="84" t="n">
         <v>-0</v>
@@ -6906,7 +6906,7 @@
         <v>99774.42999999999</v>
       </c>
       <c r="V80" s="91" t="n">
-        <v>-203.7849271649868</v>
+        <v>-206.4133332362132</v>
       </c>
       <c r="W80" s="75" t="n"/>
     </row>
@@ -6967,7 +6967,7 @@
         <v>0</v>
       </c>
       <c r="R81" s="91" t="n">
-        <v>29654.00077079122</v>
+        <v>28675.17327915017</v>
       </c>
       <c r="S81" s="84" t="n">
         <v>0</v>
@@ -7040,7 +7040,7 @@
         <v>0</v>
       </c>
       <c r="R82" s="91" t="n">
-        <v>-70354.22922920878</v>
+        <v>-71333.05672084983</v>
       </c>
       <c r="S82" s="84" t="n">
         <v>-1500123.45</v>
@@ -7113,7 +7113,7 @@
         <v>219.69</v>
       </c>
       <c r="R83" s="91" t="n">
-        <v>-70354.22922920878</v>
+        <v>-71333.05672084983</v>
       </c>
       <c r="S83" s="84" t="n">
         <v>-3006837.6</v>
@@ -7186,7 +7186,7 @@
         <v>440.83</v>
       </c>
       <c r="R84" s="91" t="n">
-        <v>-70354.22922920878</v>
+        <v>-71333.05672084983</v>
       </c>
       <c r="S84" s="84" t="n">
         <v>-3120731.25</v>
@@ -7259,7 +7259,7 @@
         <v>457.56</v>
       </c>
       <c r="R85" s="91" t="n">
-        <v>-70354.22922920878</v>
+        <v>-71333.05672084983</v>
       </c>
       <c r="S85" s="84" t="n">
         <v>-1719147.27</v>
@@ -7329,10 +7329,10 @@
         <v>0</v>
       </c>
       <c r="Q86" s="83" t="n">
-        <v>255.9</v>
+        <v>0</v>
       </c>
       <c r="R86" s="91" t="n">
-        <v>-70354.22922920878</v>
+        <v>-71588.95672084982</v>
       </c>
       <c r="S86" s="84" t="n">
         <v>-0</v>
@@ -7402,10 +7402,10 @@
         <v>0</v>
       </c>
       <c r="Q87" s="83" t="n">
-        <v>74.29000000000001</v>
+        <v>0</v>
       </c>
       <c r="R87" s="91" t="n">
-        <v>-70354.22922920878</v>
+        <v>-71663.24672084981</v>
       </c>
       <c r="S87" s="84" t="n">
         <v>-1420391</v>
@@ -7478,7 +7478,7 @@
         <v>460.31</v>
       </c>
       <c r="R88" s="91" t="n">
-        <v>-70354.22922920878</v>
+        <v>-71663.24672084981</v>
       </c>
       <c r="S88" s="84" t="n">
         <v>-3057504.3</v>
@@ -7551,7 +7551,7 @@
         <v>448.25</v>
       </c>
       <c r="R89" s="91" t="n">
-        <v>-70354.22922920878</v>
+        <v>-71663.24672084981</v>
       </c>
       <c r="S89" s="84" t="n">
         <v>-3173316.86</v>
@@ -7624,7 +7624,7 @@
         <v>465.27</v>
       </c>
       <c r="R90" s="91" t="n">
-        <v>-70354.22922920878</v>
+        <v>-71663.24672084981</v>
       </c>
       <c r="S90" s="84" t="n">
         <v>-3084909.9</v>
@@ -7697,7 +7697,7 @@
         <v>452.27</v>
       </c>
       <c r="R91" s="91" t="n">
-        <v>-70354.22922920878</v>
+        <v>-71663.24672084981</v>
       </c>
       <c r="S91" s="84" t="n">
         <v>-3201760.6</v>
@@ -7770,7 +7770,7 @@
         <v>469.44</v>
       </c>
       <c r="R92" s="91" t="n">
-        <v>-70354.22922920878</v>
+        <v>-71663.24672084981</v>
       </c>
       <c r="S92" s="84" t="n">
         <v>-3216313.24</v>
@@ -7843,7 +7843,7 @@
         <v>472.87</v>
       </c>
       <c r="R93" s="91" t="n">
-        <v>-70354.22922920878</v>
+        <v>-71663.24672084981</v>
       </c>
       <c r="S93" s="84" t="n">
         <v>-312674.73</v>
@@ -7916,7 +7916,7 @@
         <v>730.62</v>
       </c>
       <c r="R94" s="91" t="n">
-        <v>-70354.22922920878</v>
+        <v>-71663.24672084981</v>
       </c>
       <c r="S94" s="84" t="n">
         <v>-0</v>
@@ -7989,7 +7989,7 @@
         <v>45.88</v>
       </c>
       <c r="R95" s="91" t="n">
-        <v>-70354.22922920878</v>
+        <v>-71663.24672084981</v>
       </c>
       <c r="S95" s="84" t="n">
         <v>-0</v>
@@ -8062,7 +8062,7 @@
         <v>0</v>
       </c>
       <c r="R96" s="91" t="n">
-        <v>-72454.25922920878</v>
+        <v>-73763.27672084981</v>
       </c>
       <c r="S96" s="84" t="n">
         <v>-0</v>

</xml_diff>

<commit_message>
corrigindo a entrada dos xlsx na pasta out_root
</commit_message>
<xml_diff>
--- a/relatorio_final.xlsx
+++ b/relatorio_final.xlsx
@@ -1398,7 +1398,7 @@
     <row r="1">
       <c r="A1" s="135" t="inlineStr">
         <is>
-          <t>Recálculo da operação nº 145.789.000-10 - Capitalização Afastada</t>
+          <t>Recálculo da operação nº 156.789.799-10 - Capitalização Afastada</t>
         </is>
       </c>
       <c r="B1" s="30" t="n"/>
@@ -1521,7 +1521,7 @@
         </is>
       </c>
       <c r="B3" s="44" t="n">
-        <v>80000</v>
+        <v>15000</v>
       </c>
       <c r="C3" s="137" t="inlineStr">
         <is>
@@ -1578,7 +1578,7 @@
         </is>
       </c>
       <c r="D4" s="49" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E4" s="50" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
ajuste nas informações de estornos e garantias
</commit_message>
<xml_diff>
--- a/relatorio_final.xlsx
+++ b/relatorio_final.xlsx
@@ -1398,7 +1398,7 @@
     <row r="1">
       <c r="A1" s="135" t="inlineStr">
         <is>
-          <t>Recálculo da operação nº 156.789.799-10 - Capitalização Afastada</t>
+          <t>Recálculo da operação nº 145.899.700-10 - Capitalização Afastada</t>
         </is>
       </c>
       <c r="B1" s="30" t="n"/>
@@ -7913,10 +7913,10 @@
         <v>0</v>
       </c>
       <c r="Q94" s="83" t="n">
-        <v>730.62</v>
+        <v>0</v>
       </c>
       <c r="R94" s="91" t="n">
-        <v>-71663.24672084981</v>
+        <v>-72393.86672084981</v>
       </c>
       <c r="S94" s="84" t="n">
         <v>-0</v>
@@ -7989,7 +7989,7 @@
         <v>45.88</v>
       </c>
       <c r="R95" s="91" t="n">
-        <v>-71663.24672084981</v>
+        <v>-72393.86672084981</v>
       </c>
       <c r="S95" s="84" t="n">
         <v>-0</v>
@@ -8062,7 +8062,7 @@
         <v>0</v>
       </c>
       <c r="R96" s="91" t="n">
-        <v>-73763.27672084981</v>
+        <v>-74493.89672084981</v>
       </c>
       <c r="S96" s="84" t="n">
         <v>-0</v>

</xml_diff>

<commit_message>
ajustes no plan-xlsx - hitorico de estornos, renomear historico
</commit_message>
<xml_diff>
--- a/relatorio_final.xlsx
+++ b/relatorio_final.xlsx
@@ -1398,7 +1398,7 @@
     <row r="1">
       <c r="A1" s="135" t="inlineStr">
         <is>
-          <t>Recálculo da operação nº 156.489.788-10 - Capitalização Afastada</t>
+          <t>Recálculo da operação nº 897.789.889-4 - Capitalização Afastada</t>
         </is>
       </c>
       <c r="B1" s="30" t="n"/>
@@ -1521,7 +1521,7 @@
         </is>
       </c>
       <c r="B3" s="44" t="n">
-        <v>5600</v>
+        <v>560000</v>
       </c>
       <c r="C3" s="137" t="inlineStr">
         <is>
@@ -1578,7 +1578,7 @@
         </is>
       </c>
       <c r="D4" s="49" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E4" s="50" t="inlineStr">
         <is>
@@ -2511,10 +2511,10 @@
         <v>0</v>
       </c>
       <c r="Q20" s="83" t="n">
-        <v>0</v>
+        <v>305.66</v>
       </c>
       <c r="R20" s="91" t="n">
-        <v>-56547.16</v>
+        <v>-56241.5</v>
       </c>
       <c r="S20" s="84" t="n">
         <v>-0</v>
@@ -2584,10 +2584,10 @@
         <v>0</v>
       </c>
       <c r="Q21" s="83" t="n">
-        <v>0</v>
+        <v>88.73999999999999</v>
       </c>
       <c r="R21" s="91" t="n">
-        <v>-56635.9</v>
+        <v>-56241.5</v>
       </c>
       <c r="S21" s="84" t="n">
         <v>-0</v>
@@ -2660,7 +2660,7 @@
         <v>0</v>
       </c>
       <c r="R22" s="91" t="n">
-        <v>-56637.06</v>
+        <v>-56242.66</v>
       </c>
       <c r="S22" s="84" t="n">
         <v>-0</v>
@@ -2733,7 +2733,7 @@
         <v>0</v>
       </c>
       <c r="R23" s="91" t="n">
-        <v>-56637.4</v>
+        <v>-56243</v>
       </c>
       <c r="S23" s="84" t="n">
         <v>-0</v>
@@ -2806,7 +2806,7 @@
         <v>0</v>
       </c>
       <c r="R24" s="91" t="n">
-        <v>-56636.24</v>
+        <v>-56241.84</v>
       </c>
       <c r="S24" s="84" t="n">
         <v>-0</v>
@@ -2879,7 +2879,7 @@
         <v>0</v>
       </c>
       <c r="R25" s="91" t="n">
-        <v>-56635.9</v>
+        <v>-56241.5</v>
       </c>
       <c r="S25" s="84" t="n">
         <v>-0</v>
@@ -2952,7 +2952,7 @@
         <v>0</v>
       </c>
       <c r="R26" s="91" t="n">
-        <v>-96635.89999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S26" s="84" t="n">
         <v>-0</v>
@@ -3025,7 +3025,7 @@
         <v>0</v>
       </c>
       <c r="R27" s="91" t="n">
-        <v>-96787.89999999999</v>
+        <v>-96393.5</v>
       </c>
       <c r="S27" s="84" t="n">
         <v>-0</v>
@@ -3098,7 +3098,7 @@
         <v>0</v>
       </c>
       <c r="R28" s="91" t="n">
-        <v>-96635.89999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S28" s="84" t="n">
         <v>-1546174.4</v>
@@ -3171,7 +3171,7 @@
         <v>243.61</v>
       </c>
       <c r="R29" s="91" t="n">
-        <v>-96635.89999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S29" s="84" t="n">
         <v>-2906385.3</v>
@@ -3183,7 +3183,7 @@
         <v>92147.63333333333</v>
       </c>
       <c r="V29" s="91" t="n">
-        <v>-251.7414155233643</v>
+        <v>-250.7836595524696</v>
       </c>
       <c r="W29" s="75" t="n"/>
     </row>
@@ -3244,7 +3244,7 @@
         <v>427.27</v>
       </c>
       <c r="R30" s="91" t="n">
-        <v>-96635.89999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S30" s="84" t="n">
         <v>-3016510.18</v>
@@ -3256,7 +3256,7 @@
         <v>96879.50999999999</v>
       </c>
       <c r="V30" s="91" t="n">
-        <v>-426.1956010409145</v>
+        <v>-424.4561693695529</v>
       </c>
       <c r="W30" s="75" t="n"/>
     </row>
@@ -3317,7 +3317,7 @@
         <v>443.49</v>
       </c>
       <c r="R31" s="91" t="n">
-        <v>-96635.89999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S31" s="84" t="n">
         <v>-2932508.1</v>
@@ -3329,7 +3329,7 @@
         <v>97306.78</v>
       </c>
       <c r="V31" s="91" t="n">
-        <v>-455.1479644328822</v>
+        <v>-453.2903695103708</v>
       </c>
       <c r="W31" s="75" t="n"/>
     </row>
@@ -3390,7 +3390,7 @@
         <v>431.11</v>
       </c>
       <c r="R32" s="91" t="n">
-        <v>-96635.89999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S32" s="84" t="n">
         <v>-3043622.78</v>
@@ -3402,7 +3402,7 @@
         <v>97750.27</v>
       </c>
       <c r="V32" s="91" t="n">
-        <v>-426.1952713685529</v>
+        <v>-424.4558410426828</v>
       </c>
       <c r="W32" s="75" t="n"/>
     </row>
@@ -3463,7 +3463,7 @@
         <v>447.48</v>
       </c>
       <c r="R33" s="91" t="n">
-        <v>-96635.89999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S33" s="84" t="n">
         <v>-3057494.66</v>
@@ -3475,7 +3475,7 @@
         <v>98181.38</v>
       </c>
       <c r="V33" s="91" t="n">
-        <v>-455.1519127992948</v>
+        <v>-453.2943017623195</v>
       </c>
       <c r="W33" s="75" t="n"/>
     </row>
@@ -3536,7 +3536,7 @@
         <v>449.52</v>
       </c>
       <c r="R34" s="91" t="n">
-        <v>-96635.89999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S34" s="84" t="n">
         <v>-2774194.64</v>
@@ -3548,7 +3548,7 @@
         <v>98628.86</v>
       </c>
       <c r="V34" s="91" t="n">
-        <v>-455.1524456510132</v>
+        <v>-453.2948324393108</v>
       </c>
       <c r="W34" s="75" t="n"/>
     </row>
@@ -3609,7 +3609,7 @@
         <v>407.78</v>
       </c>
       <c r="R35" s="91" t="n">
-        <v>-96635.89999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S35" s="84" t="n">
         <v>-3084070.96</v>
@@ -3621,7 +3621,7 @@
         <v>99078.38</v>
       </c>
       <c r="V35" s="91" t="n">
-        <v>-371.16139517371</v>
+        <v>-369.6465745505615</v>
       </c>
       <c r="W35" s="75" t="n"/>
     </row>
@@ -3682,7 +3682,7 @@
         <v>453.42</v>
       </c>
       <c r="R36" s="91" t="n">
-        <v>-96635.89999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S36" s="84" t="n">
         <v>-2998187.4</v>
@@ -3694,7 +3694,7 @@
         <v>99486.16</v>
       </c>
       <c r="V36" s="91" t="n">
-        <v>-455.1451076391307</v>
+        <v>-453.2875243760486</v>
       </c>
       <c r="W36" s="75" t="n"/>
     </row>
@@ -3755,7 +3755,7 @@
         <v>440.76</v>
       </c>
       <c r="R37" s="91" t="n">
-        <v>-96635.89999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S37" s="84" t="n">
         <v>-3111790.54</v>
@@ -3767,7 +3767,7 @@
         <v>99939.58</v>
       </c>
       <c r="V37" s="91" t="n">
-        <v>-426.1898967756351</v>
+        <v>-424.4504883850855</v>
       </c>
       <c r="W37" s="75" t="n"/>
     </row>
@@ -3828,7 +3828,7 @@
         <v>457.5</v>
       </c>
       <c r="R38" s="91" t="n">
-        <v>-96635.89999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S38" s="84" t="n">
         <v>-3025135.2</v>
@@ -3840,7 +3840,7 @@
         <v>100380.34</v>
       </c>
       <c r="V38" s="91" t="n">
-        <v>-455.1497523686898</v>
+        <v>-453.2921501490778</v>
       </c>
       <c r="W38" s="75" t="n"/>
     </row>
@@ -3901,7 +3901,7 @@
         <v>444.73</v>
       </c>
       <c r="R39" s="91" t="n">
-        <v>-96635.89999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S39" s="84" t="n">
         <v>-3139759.67</v>
@@ -3913,7 +3913,7 @@
         <v>100837.84</v>
       </c>
       <c r="V39" s="91" t="n">
-        <v>-426.197980906763</v>
+        <v>-424.4585395224573</v>
       </c>
       <c r="W39" s="75" t="n"/>
     </row>
@@ -3974,7 +3974,7 @@
         <v>461.61</v>
       </c>
       <c r="R40" s="91" t="n">
-        <v>-96635.89999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S40" s="84" t="n">
         <v>-2034883.6</v>
@@ -3986,7 +3986,7 @@
         <v>101282.57</v>
       </c>
       <c r="V40" s="91" t="n">
-        <v>-455.1477186558352</v>
+        <v>-453.2901247364134</v>
       </c>
       <c r="W40" s="75" t="n"/>
     </row>
@@ -4044,10 +4044,10 @@
         <v>0</v>
       </c>
       <c r="Q41" s="83" t="n">
-        <v>0</v>
+        <v>279.67</v>
       </c>
       <c r="R41" s="91" t="n">
-        <v>-96915.56999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S41" s="84" t="n">
         <v>-0</v>
@@ -4117,10 +4117,10 @@
         <v>0</v>
       </c>
       <c r="Q42" s="83" t="n">
-        <v>0</v>
+        <v>81.19</v>
       </c>
       <c r="R42" s="91" t="n">
-        <v>-96996.75999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S42" s="84" t="n">
         <v>-0</v>
@@ -4193,7 +4193,7 @@
         <v>0</v>
       </c>
       <c r="R43" s="91" t="n">
-        <v>-96997.81999999999</v>
+        <v>-96242.56</v>
       </c>
       <c r="S43" s="84" t="n">
         <v>-0</v>
@@ -4266,7 +4266,7 @@
         <v>0</v>
       </c>
       <c r="R44" s="91" t="n">
-        <v>-96998.12999999999</v>
+        <v>-96242.87</v>
       </c>
       <c r="S44" s="84" t="n">
         <v>-0</v>
@@ -4339,7 +4339,7 @@
         <v>0</v>
       </c>
       <c r="R45" s="91" t="n">
-        <v>-96997.06999999999</v>
+        <v>-96241.81</v>
       </c>
       <c r="S45" s="84" t="n">
         <v>-0</v>
@@ -4412,7 +4412,7 @@
         <v>0</v>
       </c>
       <c r="R46" s="91" t="n">
-        <v>-96996.75999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S46" s="84" t="n">
         <v>-1123155.44</v>
@@ -4485,7 +4485,7 @@
         <v>464.3</v>
       </c>
       <c r="R47" s="91" t="n">
-        <v>-96996.75999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S47" s="84" t="n">
         <v>-3077080.2</v>
@@ -4497,7 +4497,7 @@
         <v>101872.2270967742</v>
       </c>
       <c r="V47" s="91" t="n">
-        <v>-455.7533161977407</v>
+        <v>-453.2926166909854</v>
       </c>
       <c r="W47" s="75" t="n"/>
     </row>
@@ -4558,7 +4558,7 @@
         <v>452.36</v>
       </c>
       <c r="R48" s="91" t="n">
-        <v>-96996.75999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S48" s="84" t="n">
         <v>-3193672.7</v>
@@ -4570,7 +4570,7 @@
         <v>102569.34</v>
       </c>
       <c r="V48" s="91" t="n">
-        <v>-427.7833351915854</v>
+        <v>-424.4524235019908</v>
       </c>
       <c r="W48" s="75" t="n"/>
     </row>
@@ -4631,7 +4631,7 @@
         <v>469.54</v>
       </c>
       <c r="R49" s="91" t="n">
-        <v>-96996.75999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S49" s="84" t="n">
         <v>-3104737.2</v>
@@ -4643,7 +4643,7 @@
         <v>103021.7</v>
       </c>
       <c r="V49" s="91" t="n">
-        <v>-456.8509058466366</v>
+        <v>-453.2936610979489</v>
       </c>
       <c r="W49" s="75" t="n"/>
     </row>
@@ -4704,7 +4704,7 @@
         <v>456.43</v>
       </c>
       <c r="R50" s="91" t="n">
-        <v>-96996.75999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S50" s="84" t="n">
         <v>-3222377.77</v>
@@ -4716,7 +4716,7 @@
         <v>103491.24</v>
       </c>
       <c r="V50" s="91" t="n">
-        <v>-427.7872326855828</v>
+        <v>-424.4562906483631</v>
       </c>
       <c r="W50" s="75" t="n"/>
     </row>
@@ -4777,7 +4777,7 @@
         <v>473.76</v>
       </c>
       <c r="R51" s="91" t="n">
-        <v>-96996.75999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S51" s="84" t="n">
         <v>-3237064.33</v>
@@ -4789,7 +4789,7 @@
         <v>103947.67</v>
       </c>
       <c r="V51" s="91" t="n">
-        <v>-456.8506401846879</v>
+        <v>-453.2933975045624</v>
       </c>
       <c r="W51" s="75" t="n"/>
     </row>
@@ -4850,7 +4850,7 @@
         <v>475.92</v>
       </c>
       <c r="R52" s="91" t="n">
-        <v>-96996.75999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S52" s="84" t="n">
         <v>-2937125.8</v>
@@ -4862,7 +4862,7 @@
         <v>104421.43</v>
       </c>
       <c r="V52" s="91" t="n">
-        <v>-456.8513645190588</v>
+        <v>-453.2941161989432</v>
       </c>
       <c r="W52" s="75" t="n"/>
     </row>
@@ -4923,7 +4923,7 @@
         <v>431.72</v>
       </c>
       <c r="R53" s="91" t="n">
-        <v>-96996.75999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S53" s="84" t="n">
         <v>-3265201.17</v>
@@ -4935,7 +4935,7 @@
         <v>104897.35</v>
       </c>
       <c r="V53" s="91" t="n">
-        <v>-372.5393553862689</v>
+        <v>-369.6385979429375</v>
       </c>
       <c r="W53" s="75" t="n"/>
     </row>
@@ -4996,7 +4996,7 @@
         <v>480.05</v>
       </c>
       <c r="R54" s="91" t="n">
-        <v>-96996.75999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S54" s="84" t="n">
         <v>-3174273.6</v>
@@ -5008,7 +5008,7 @@
         <v>105329.07</v>
       </c>
       <c r="V54" s="91" t="n">
-        <v>-456.8449523664911</v>
+        <v>-453.2877539742529</v>
       </c>
       <c r="W54" s="75" t="n"/>
     </row>
@@ -5069,7 +5069,7 @@
         <v>466.65</v>
       </c>
       <c r="R55" s="91" t="n">
-        <v>-96996.75999999999</v>
+        <v>-96241.5</v>
       </c>
       <c r="S55" s="84" t="n">
         <v>-1700412.32</v>
@@ -5081,7 +5081,7 @@
         <v>105809.12</v>
       </c>
       <c r="V55" s="91" t="n">
-        <v>-427.7848455218292</v>
+        <v>-424.4539220721303</v>
       </c>
       <c r="W55" s="75" t="n"/>
     </row>
@@ -5142,7 +5142,7 @@
         <v>0</v>
       </c>
       <c r="R56" s="91" t="n">
-        <v>-96937.84</v>
+        <v>-96182.58</v>
       </c>
       <c r="S56" s="84" t="n">
         <v>-1168385.35</v>
@@ -5215,7 +5215,7 @@
         <v>0</v>
       </c>
       <c r="R57" s="91" t="n">
-        <v>-96853.92999999999</v>
+        <v>-96098.67</v>
       </c>
       <c r="S57" s="84" t="n">
         <v>-0</v>
@@ -5288,7 +5288,7 @@
         <v>0</v>
       </c>
       <c r="R58" s="91" t="n">
-        <v>-90604.87</v>
+        <v>-89849.61</v>
       </c>
       <c r="S58" s="84" t="n">
         <v>-0</v>
@@ -5361,7 +5361,7 @@
         <v>0</v>
       </c>
       <c r="R59" s="91" t="n">
-        <v>-89896.33</v>
+        <v>-89141.07000000001</v>
       </c>
       <c r="S59" s="84" t="n">
         <v>-0</v>
@@ -5434,7 +5434,7 @@
         <v>0</v>
       </c>
       <c r="R60" s="91" t="n">
-        <v>-85451.89</v>
+        <v>-84696.63</v>
       </c>
       <c r="S60" s="84" t="n">
         <v>-0</v>
@@ -5507,7 +5507,7 @@
         <v>0</v>
       </c>
       <c r="R61" s="91" t="n">
-        <v>-84912.10000000001</v>
+        <v>-84156.84000000001</v>
       </c>
       <c r="S61" s="84" t="n">
         <v>-376764.44</v>
@@ -5580,7 +5580,7 @@
         <v>477.18</v>
       </c>
       <c r="R62" s="91" t="n">
-        <v>-84912.10000000001</v>
+        <v>-84156.84000000001</v>
       </c>
       <c r="S62" s="84" t="n">
         <v>-2840048.7</v>
@@ -5592,7 +5592,7 @@
         <v>104695.5519354839</v>
       </c>
       <c r="V62" s="91" t="n">
-        <v>-449.4186127781232</v>
+        <v>-445.8612851428762</v>
       </c>
       <c r="W62" s="75" t="n"/>
     </row>
@@ -5653,7 +5653,7 @@
         <v>417.52</v>
       </c>
       <c r="R63" s="91" t="n">
-        <v>-84912.10000000001</v>
+        <v>-84156.84000000001</v>
       </c>
       <c r="S63" s="84" t="n">
         <v>-2947660.11</v>
@@ -5665,7 +5665,7 @@
         <v>94668.28999999999</v>
       </c>
       <c r="V63" s="91" t="n">
-        <v>-374.491817608628</v>
+        <v>-371.1608590035871</v>
       </c>
       <c r="W63" s="75" t="n"/>
     </row>
@@ -5726,7 +5726,7 @@
         <v>433.37</v>
       </c>
       <c r="R64" s="91" t="n">
-        <v>-84912.10000000001</v>
+        <v>-84156.84000000001</v>
       </c>
       <c r="S64" s="84" t="n">
         <v>-1814864.42</v>
@@ -5738,7 +5738,7 @@
         <v>95085.81</v>
       </c>
       <c r="V64" s="91" t="n">
-        <v>-399.9319442075342</v>
+        <v>-396.3747056021743</v>
       </c>
       <c r="W64" s="75" t="n"/>
     </row>
@@ -5796,10 +5796,10 @@
         <v>0</v>
       </c>
       <c r="Q65" s="83" t="n">
-        <v>0</v>
+        <v>255.9</v>
       </c>
       <c r="R65" s="91" t="n">
-        <v>-85168</v>
+        <v>-84156.84000000001</v>
       </c>
       <c r="S65" s="84" t="n">
         <v>-0</v>
@@ -5869,10 +5869,10 @@
         <v>0</v>
       </c>
       <c r="Q66" s="83" t="n">
-        <v>0</v>
+        <v>74.29000000000001</v>
       </c>
       <c r="R66" s="91" t="n">
-        <v>-85242.28999999999</v>
+        <v>-84156.84000000001</v>
       </c>
       <c r="S66" s="84" t="n">
         <v>-0</v>
@@ -5945,7 +5945,7 @@
         <v>0</v>
       </c>
       <c r="R67" s="91" t="n">
-        <v>-85243.25999999999</v>
+        <v>-84157.81000000001</v>
       </c>
       <c r="S67" s="84" t="n">
         <v>-0</v>
@@ -6018,7 +6018,7 @@
         <v>0</v>
       </c>
       <c r="R68" s="91" t="n">
-        <v>-85243.53999999999</v>
+        <v>-84158.09000000001</v>
       </c>
       <c r="S68" s="84" t="n">
         <v>-0</v>
@@ -6091,7 +6091,7 @@
         <v>0</v>
       </c>
       <c r="R69" s="91" t="n">
-        <v>-85242.56999999999</v>
+        <v>-84157.12000000001</v>
       </c>
       <c r="S69" s="84" t="n">
         <v>-0</v>
@@ -6164,7 +6164,7 @@
         <v>0</v>
       </c>
       <c r="R70" s="91" t="n">
-        <v>-85242.28999999999</v>
+        <v>-84156.84000000001</v>
       </c>
       <c r="S70" s="84" t="n">
         <v>-1150192.44</v>
@@ -6237,7 +6237,7 @@
         <v>435.92</v>
       </c>
       <c r="R71" s="91" t="n">
-        <v>-85242.28999999999</v>
+        <v>-84156.84000000001</v>
       </c>
       <c r="S71" s="84" t="n">
         <v>-2888558.7</v>
@@ -6249,7 +6249,7 @@
         <v>95646.99548387097</v>
       </c>
       <c r="V71" s="91" t="n">
-        <v>-400.5268739092156</v>
+        <v>-396.3677039362893</v>
       </c>
       <c r="W71" s="75" t="n"/>
     </row>
@@ -6310,7 +6310,7 @@
         <v>424.65</v>
       </c>
       <c r="R72" s="91" t="n">
-        <v>-85242.28999999999</v>
+        <v>-84156.84000000001</v>
       </c>
       <c r="S72" s="84" t="n">
         <v>-2998008.14</v>
@@ -6322,7 +6322,7 @@
         <v>96285.28999999999</v>
       </c>
       <c r="V72" s="91" t="n">
-        <v>-375.9467146902618</v>
+        <v>-371.15952089877</v>
       </c>
       <c r="W72" s="75" t="n"/>
     </row>
@@ -6383,7 +6383,7 @@
         <v>440.77</v>
       </c>
       <c r="R73" s="91" t="n">
-        <v>-85242.28999999999</v>
+        <v>-84156.84000000001</v>
       </c>
       <c r="S73" s="84" t="n">
         <v>-2914521.3</v>
@@ -6395,7 +6395,7 @@
         <v>96709.94</v>
       </c>
       <c r="V73" s="91" t="n">
-        <v>-401.4850710615175</v>
+        <v>-396.3726794260544</v>
       </c>
       <c r="W73" s="75" t="n"/>
     </row>
@@ -6456,7 +6456,7 @@
         <v>428.46</v>
       </c>
       <c r="R74" s="91" t="n">
-        <v>-85242.28999999999</v>
+        <v>-84156.84000000001</v>
       </c>
       <c r="S74" s="84" t="n">
         <v>-3024954.27</v>
@@ -6468,7 +6468,7 @@
         <v>97150.71000000001</v>
       </c>
       <c r="V74" s="91" t="n">
-        <v>-375.9407581622424</v>
+        <v>-371.1536402194092</v>
       </c>
       <c r="W74" s="75" t="n"/>
     </row>
@@ -6529,7 +6529,7 @@
         <v>444.73</v>
       </c>
       <c r="R75" s="91" t="n">
-        <v>-85242.28999999999</v>
+        <v>-84156.84000000001</v>
       </c>
       <c r="S75" s="84" t="n">
         <v>-3038740.9</v>
@@ -6541,7 +6541,7 @@
         <v>97579.17</v>
       </c>
       <c r="V75" s="91" t="n">
-        <v>-401.4835853813657</v>
+        <v>-396.3712126641124</v>
       </c>
       <c r="W75" s="75" t="n"/>
     </row>
@@ -6602,7 +6602,7 @@
         <v>445.54</v>
       </c>
       <c r="R76" s="91" t="n">
-        <v>-85242.28999999999</v>
+        <v>-84156.84000000001</v>
       </c>
       <c r="S76" s="84" t="n">
         <v>-2855613.76</v>
@@ -6614,7 +6614,7 @@
         <v>98023.89999999999</v>
       </c>
       <c r="V76" s="91" t="n">
-        <v>-400.3899063617669</v>
+        <v>-395.2914602282764</v>
       </c>
       <c r="W76" s="75" t="n"/>
     </row>
@@ -6675,7 +6675,7 @@
         <v>418.62</v>
       </c>
       <c r="R77" s="91" t="n">
-        <v>-85242.28999999999</v>
+        <v>-84156.84000000001</v>
       </c>
       <c r="S77" s="84" t="n">
         <v>-3065529.86</v>
@@ -6687,7 +6687,7 @@
         <v>98469.44</v>
       </c>
       <c r="V77" s="91" t="n">
-        <v>-350.2834584595251</v>
+        <v>-345.8230529497143</v>
       </c>
       <c r="W77" s="75" t="n"/>
     </row>
@@ -6748,7 +6748,7 @@
         <v>449.46</v>
       </c>
       <c r="R78" s="91" t="n">
-        <v>-85242.28999999999</v>
+        <v>-84156.84000000001</v>
       </c>
       <c r="S78" s="84" t="n">
         <v>-2980125.6</v>
@@ -6760,7 +6760,7 @@
         <v>98888.06</v>
       </c>
       <c r="V78" s="91" t="n">
-        <v>-400.3829614176663</v>
+        <v>-395.2846037190311</v>
       </c>
       <c r="W78" s="75" t="n"/>
     </row>
@@ -6821,7 +6821,7 @@
         <v>436.91</v>
       </c>
       <c r="R79" s="91" t="n">
-        <v>-85242.28999999999</v>
+        <v>-84156.84000000001</v>
       </c>
       <c r="S79" s="84" t="n">
         <v>-1596390.88</v>
@@ -6833,7 +6833,7 @@
         <v>99337.52</v>
       </c>
       <c r="V79" s="91" t="n">
-        <v>-374.9158316404446</v>
+        <v>-370.1417648074898</v>
       </c>
       <c r="W79" s="75" t="n"/>
     </row>
@@ -6888,13 +6888,13 @@
         </is>
       </c>
       <c r="P80" s="88" t="n">
-        <v>-13909.23327915017</v>
+        <v>-13802.61077079124</v>
       </c>
       <c r="Q80" s="83" t="n">
         <v>233.8</v>
       </c>
       <c r="R80" s="91" t="n">
-        <v>-71333.05672084983</v>
+        <v>-70354.22922920878</v>
       </c>
       <c r="S80" s="84" t="n">
         <v>-0</v>
@@ -6906,7 +6906,7 @@
         <v>99774.42999999999</v>
       </c>
       <c r="V80" s="91" t="n">
-        <v>-206.4133332362132</v>
+        <v>-203.7849271649868</v>
       </c>
       <c r="W80" s="75" t="n"/>
     </row>
@@ -6967,7 +6967,7 @@
         <v>0</v>
       </c>
       <c r="R81" s="91" t="n">
-        <v>28675.17327915017</v>
+        <v>29654.00077079122</v>
       </c>
       <c r="S81" s="84" t="n">
         <v>0</v>
@@ -7040,7 +7040,7 @@
         <v>0</v>
       </c>
       <c r="R82" s="91" t="n">
-        <v>-71333.05672084983</v>
+        <v>-70354.22922920878</v>
       </c>
       <c r="S82" s="84" t="n">
         <v>-1500123.45</v>
@@ -7113,7 +7113,7 @@
         <v>219.69</v>
       </c>
       <c r="R83" s="91" t="n">
-        <v>-71333.05672084983</v>
+        <v>-70354.22922920878</v>
       </c>
       <c r="S83" s="84" t="n">
         <v>-3006837.6</v>
@@ -7186,7 +7186,7 @@
         <v>440.83</v>
       </c>
       <c r="R84" s="91" t="n">
-        <v>-71333.05672084983</v>
+        <v>-70354.22922920878</v>
       </c>
       <c r="S84" s="84" t="n">
         <v>-3120731.25</v>
@@ -7259,7 +7259,7 @@
         <v>457.56</v>
       </c>
       <c r="R85" s="91" t="n">
-        <v>-71333.05672084983</v>
+        <v>-70354.22922920878</v>
       </c>
       <c r="S85" s="84" t="n">
         <v>-1719147.27</v>
@@ -7329,10 +7329,10 @@
         <v>0</v>
       </c>
       <c r="Q86" s="83" t="n">
-        <v>0</v>
+        <v>255.9</v>
       </c>
       <c r="R86" s="91" t="n">
-        <v>-71588.95672084982</v>
+        <v>-70354.22922920878</v>
       </c>
       <c r="S86" s="84" t="n">
         <v>-0</v>
@@ -7402,10 +7402,10 @@
         <v>0</v>
       </c>
       <c r="Q87" s="83" t="n">
-        <v>0</v>
+        <v>74.29000000000001</v>
       </c>
       <c r="R87" s="91" t="n">
-        <v>-71663.24672084981</v>
+        <v>-70354.22922920878</v>
       </c>
       <c r="S87" s="84" t="n">
         <v>-1420391</v>
@@ -7478,7 +7478,7 @@
         <v>460.31</v>
       </c>
       <c r="R88" s="91" t="n">
-        <v>-71663.24672084981</v>
+        <v>-70354.22922920878</v>
       </c>
       <c r="S88" s="84" t="n">
         <v>-3057504.3</v>
@@ -7551,7 +7551,7 @@
         <v>448.25</v>
       </c>
       <c r="R89" s="91" t="n">
-        <v>-71663.24672084981</v>
+        <v>-70354.22922920878</v>
       </c>
       <c r="S89" s="84" t="n">
         <v>-3173316.86</v>
@@ -7624,7 +7624,7 @@
         <v>465.27</v>
       </c>
       <c r="R90" s="91" t="n">
-        <v>-71663.24672084981</v>
+        <v>-70354.22922920878</v>
       </c>
       <c r="S90" s="84" t="n">
         <v>-3084909.9</v>
@@ -7697,7 +7697,7 @@
         <v>452.27</v>
       </c>
       <c r="R91" s="91" t="n">
-        <v>-71663.24672084981</v>
+        <v>-70354.22922920878</v>
       </c>
       <c r="S91" s="84" t="n">
         <v>-3201760.6</v>
@@ -7770,7 +7770,7 @@
         <v>469.44</v>
       </c>
       <c r="R92" s="91" t="n">
-        <v>-71663.24672084981</v>
+        <v>-70354.22922920878</v>
       </c>
       <c r="S92" s="84" t="n">
         <v>-3216313.24</v>
@@ -7843,7 +7843,7 @@
         <v>472.87</v>
       </c>
       <c r="R93" s="91" t="n">
-        <v>-71663.24672084981</v>
+        <v>-70354.22922920878</v>
       </c>
       <c r="S93" s="84" t="n">
         <v>-312674.73</v>
@@ -7916,7 +7916,7 @@
         <v>0</v>
       </c>
       <c r="R94" s="91" t="n">
-        <v>-72393.86672084981</v>
+        <v>-71084.84922920878</v>
       </c>
       <c r="S94" s="84" t="n">
         <v>-0</v>
@@ -7989,7 +7989,7 @@
         <v>45.88</v>
       </c>
       <c r="R95" s="91" t="n">
-        <v>-72393.86672084981</v>
+        <v>-71084.84922920878</v>
       </c>
       <c r="S95" s="84" t="n">
         <v>-0</v>
@@ -8062,7 +8062,7 @@
         <v>0</v>
       </c>
       <c r="R96" s="91" t="n">
-        <v>-74493.89672084981</v>
+        <v>-73184.87922920877</v>
       </c>
       <c r="S96" s="84" t="n">
         <v>-0</v>

</xml_diff>